<commit_message>
Remove photo upload button
</commit_message>
<xml_diff>
--- a/japantour.xlsx
+++ b/japantour.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30509"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30502"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bscvn-my.sharepoint.com/personal/minhpq_bsc_com_vn/Documents/09_CODER/00_travel-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="51" documentId="13_ncr:1_{4CBA3FCD-3F21-4F99-9320-E2DF1148D8FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51FDC033-B0FC-4F59-9377-7088DF886B9E}"/>
+  <xr:revisionPtr revIDLastSave="80" documentId="13_ncr:1_{4CBA3FCD-3F21-4F99-9320-E2DF1148D8FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{314FF19D-E644-4827-A62E-DD14149C9AEB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="458" firstSheet="4" activeTab="4" xr2:uid="{1D34A874-FA64-408A-8A73-D0DA492D543E}"/>
   </bookViews>
@@ -1385,16 +1385,17 @@
     <t>On Flight</t>
   </si>
   <si>
-    <t>Depart HAN on flight VJ 932 to NRT from HAN</t>
+    <t>Depart HAN on flight VJ 932 to NRT</t>
   </si>
   <si>
     <t>08:00 - 11:00</t>
   </si>
   <si>
-    <t>Arrival &amp; Immigration</t>
-  </si>
-  <si>
-    <t>Complete immigration and Send Luggage at Narita Airport.</t>
+    <t>Send Luggage</t>
+  </si>
+  <si>
+    <t>Send Luggage at Yamato Transport
+(Terminal 2, 3rd Floor)</t>
   </si>
   <si>
     <t>11:00 - 12:00</t>
@@ -1403,7 +1404,8 @@
     <t>Airport Transfer</t>
   </si>
   <si>
-    <t>Transfer from Narita Airport to Tokyo (Ota-ku / Heiwajima) via Keisei Skyliner / Train.</t>
+    <t>Transfer from Narita Airport to Tokyo (Ota-ku / Heiwajima) via Keisei Skyliner / Train
+(Airbnb address: https://maps.app.goo.gl/DBmdvffro3LetJej6)</t>
   </si>
   <si>
     <t>12:00 - 13:00</t>
@@ -1744,7 +1746,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="35">
+  <fonts count="33">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1958,51 +1960,32 @@
     </font>
     <font>
       <b/>
-      <sz val="9"/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Aptos Display"/>
-      <family val="2"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FF123056"/>
-      <name val="Aptos Display"/>
-      <family val="2"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Aptos Display"/>
-      <family val="2"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF333333"/>
-      <name val="Aptos Display"/>
-      <family val="2"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF222222"/>
-      <name val="Aptos Display"/>
-      <family val="2"/>
-      <scheme val="major"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="0"/>
-      <name val="Aptos Display"/>
-      <family val="2"/>
-      <scheme val="major"/>
+      <color rgb="FF123056"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF333333"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF222222"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2057,8 +2040,14 @@
         <bgColor rgb="FFF9FBFD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -2164,13 +2153,41 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7DE"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7DE"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D7DE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7DE"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7DE"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD0D7DE"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="255">
+  <cellXfs count="263">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2812,30 +2829,51 @@
     <xf numFmtId="0" fontId="29" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="20" fontId="32" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="31" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -2860,8 +2898,9 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
@@ -5937,7 +5976,7 @@
     <row r="137" spans="1:8" ht="15" customHeight="1">
       <c r="A137" s="37"/>
       <c r="B137" s="38"/>
-      <c r="C137" s="245" t="s">
+      <c r="C137" s="252" t="s">
         <v>179</v>
       </c>
       <c r="D137" s="38"/>
@@ -5952,7 +5991,7 @@
     <row r="138" spans="1:8" ht="15" customHeight="1">
       <c r="A138" s="37"/>
       <c r="B138" s="38"/>
-      <c r="C138" s="245"/>
+      <c r="C138" s="252"/>
       <c r="D138" s="38"/>
       <c r="E138" s="39"/>
       <c r="F138" s="38"/>
@@ -6678,8 +6717,8 @@
         <v>225</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="246" customFormat="1">
-      <c r="A2" s="246" t="s">
+    <row r="2" spans="1:10" s="253" customFormat="1">
+      <c r="A2" s="253" t="s">
         <v>226</v>
       </c>
     </row>
@@ -6786,10 +6825,10 @@
     <row r="8" spans="1:10">
       <c r="A8" s="84"/>
       <c r="B8" s="85"/>
-      <c r="C8" s="247" t="s">
+      <c r="C8" s="254" t="s">
         <v>230</v>
       </c>
-      <c r="D8" s="247"/>
+      <c r="D8" s="254"/>
       <c r="E8" s="96">
         <v>1500</v>
       </c>
@@ -6832,10 +6871,10 @@
       <c r="J10" s="85"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="247" t="s">
+      <c r="A11" s="254" t="s">
         <v>233</v>
       </c>
-      <c r="B11" s="247"/>
+      <c r="B11" s="254"/>
       <c r="C11" s="99">
         <v>27</v>
       </c>
@@ -9169,8 +9208,8 @@
         <v>225</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="246" customFormat="1">
-      <c r="A2" s="246" t="s">
+    <row r="2" spans="1:12" s="253" customFormat="1">
+      <c r="A2" s="253" t="s">
         <v>226</v>
       </c>
     </row>
@@ -9331,10 +9370,10 @@
     <row r="10" spans="1:12">
       <c r="A10" s="84"/>
       <c r="B10" s="85"/>
-      <c r="C10" s="247" t="s">
+      <c r="C10" s="254" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="247"/>
+      <c r="D10" s="254"/>
       <c r="E10" s="96">
         <v>3000</v>
       </c>
@@ -9377,10 +9416,10 @@
       <c r="J12" s="85"/>
     </row>
     <row r="13" spans="1:12">
-      <c r="A13" s="247" t="s">
+      <c r="A13" s="254" t="s">
         <v>233</v>
       </c>
-      <c r="B13" s="247"/>
+      <c r="B13" s="254"/>
       <c r="C13" s="99">
         <v>13</v>
       </c>
@@ -9804,10 +9843,10 @@
     <row r="34" spans="1:12">
       <c r="A34" s="114"/>
       <c r="B34" s="127"/>
-      <c r="C34" s="249" t="s">
+      <c r="C34" s="256" t="s">
         <v>338</v>
       </c>
-      <c r="D34" s="249"/>
+      <c r="D34" s="256"/>
       <c r="E34" s="128"/>
       <c r="F34" s="129"/>
       <c r="G34" s="127"/>
@@ -9820,10 +9859,10 @@
     <row r="35" spans="1:12">
       <c r="A35" s="114"/>
       <c r="B35" s="127"/>
-      <c r="C35" s="250" t="s">
+      <c r="C35" s="257" t="s">
         <v>50</v>
       </c>
-      <c r="D35" s="250"/>
+      <c r="D35" s="257"/>
       <c r="E35" s="128"/>
       <c r="F35" s="129"/>
       <c r="G35" s="127"/>
@@ -9840,10 +9879,10 @@
       <c r="B36" s="101">
         <v>0.33333333333333331</v>
       </c>
-      <c r="C36" s="252" t="s">
+      <c r="C36" s="259" t="s">
         <v>51</v>
       </c>
-      <c r="D36" s="252"/>
+      <c r="D36" s="259"/>
       <c r="E36" s="132"/>
       <c r="F36" s="133"/>
       <c r="G36" s="134"/>
@@ -10090,10 +10129,10 @@
     <row r="48" spans="1:12">
       <c r="A48" s="114"/>
       <c r="B48" s="109"/>
-      <c r="C48" s="251" t="s">
+      <c r="C48" s="258" t="s">
         <v>352</v>
       </c>
-      <c r="D48" s="251"/>
+      <c r="D48" s="258"/>
       <c r="E48" s="96">
         <f>370+220</f>
         <v>590</v>
@@ -10896,7 +10935,7 @@
     <row r="83" spans="1:10">
       <c r="A83" s="114"/>
       <c r="B83" s="109"/>
-      <c r="C83" s="248" t="s">
+      <c r="C83" s="255" t="s">
         <v>377</v>
       </c>
       <c r="D83" s="148" t="s">
@@ -10922,7 +10961,7 @@
     <row r="84" spans="1:10">
       <c r="A84" s="114"/>
       <c r="B84" s="109"/>
-      <c r="C84" s="248"/>
+      <c r="C84" s="255"/>
       <c r="D84" s="148" t="s">
         <v>379</v>
       </c>
@@ -12707,16 +12746,16 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18" style="10" customWidth="1"/>
-    <col min="2" max="2" width="28" style="10" customWidth="1"/>
-    <col min="3" max="3" width="81" style="10" customWidth="1"/>
-    <col min="4" max="16384" width="8.85546875" style="10"/>
+    <col min="1" max="1" width="18" style="216" customWidth="1"/>
+    <col min="2" max="2" width="28" style="216" customWidth="1"/>
+    <col min="3" max="3" width="81" style="216" customWidth="1"/>
+    <col min="4" max="16384" width="8.85546875" style="216"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:3">
       <c r="A1" s="236" t="s">
         <v>432</v>
       </c>
@@ -12726,16 +12765,15 @@
       <c r="C1" s="236" t="s">
         <v>434</v>
       </c>
-      <c r="D1" s="253"/>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="244" t="s">
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="250" t="s">
         <v>435</v>
       </c>
-      <c r="B2" s="254"/>
-      <c r="C2" s="254"/>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="B2" s="260"/>
+      <c r="C2" s="260"/>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" s="237" t="s">
         <v>436</v>
       </c>
@@ -12746,7 +12784,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:3" ht="29.25">
       <c r="A4" s="240" t="s">
         <v>439</v>
       </c>
@@ -12757,7 +12795,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:3" ht="29.25">
       <c r="A5" s="237" t="s">
         <v>442</v>
       </c>
@@ -12768,7 +12806,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:3">
       <c r="A6" s="240" t="s">
         <v>445</v>
       </c>
@@ -12779,7 +12817,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:3">
       <c r="A7" s="237" t="s">
         <v>448</v>
       </c>
@@ -12790,7 +12828,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:3">
       <c r="A8" s="240" t="s">
         <v>451</v>
       </c>
@@ -12801,7 +12839,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:3">
       <c r="A9" s="237" t="s">
         <v>454</v>
       </c>
@@ -12812,7 +12850,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:3">
       <c r="A10" s="240" t="s">
         <v>457</v>
       </c>
@@ -12823,25 +12861,25 @@
         <v>459</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A11" s="237" t="s">
+    <row r="11" spans="1:3">
+      <c r="A11" s="243" t="s">
         <v>460</v>
       </c>
-      <c r="B11" s="238" t="s">
+      <c r="B11" s="244" t="s">
         <v>461</v>
       </c>
-      <c r="C11" s="239" t="s">
+      <c r="C11" s="245" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="244" t="s">
+    <row r="12" spans="1:3">
+      <c r="A12" s="251" t="s">
         <v>463</v>
       </c>
-      <c r="B12" s="254"/>
-      <c r="C12" s="254"/>
-    </row>
-    <row r="13" spans="1:4">
+      <c r="B12" s="261"/>
+      <c r="C12" s="261"/>
+    </row>
+    <row r="13" spans="1:3">
       <c r="A13" s="237" t="s">
         <v>464</v>
       </c>
@@ -12852,7 +12890,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="24">
+    <row r="14" spans="1:3" ht="29.25">
       <c r="A14" s="240" t="s">
         <v>467</v>
       </c>
@@ -12863,7 +12901,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:3">
       <c r="A15" s="237" t="s">
         <v>470</v>
       </c>
@@ -12874,23 +12912,23 @@
         <v>471</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A16" s="243">
+    <row r="16" spans="1:3">
+      <c r="A16" s="246">
         <v>0.875</v>
       </c>
-      <c r="B16" s="241" t="s">
+      <c r="B16" s="247" t="s">
         <v>472</v>
       </c>
-      <c r="C16" s="242" t="s">
+      <c r="C16" s="248" t="s">
         <v>473</v>
       </c>
     </row>
     <row r="17" spans="1:3">
-      <c r="A17" s="244" t="s">
+      <c r="A17" s="251" t="s">
         <v>474</v>
       </c>
-      <c r="B17" s="254"/>
-      <c r="C17" s="254"/>
+      <c r="B17" s="261"/>
+      <c r="C17" s="261"/>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="237" t="s">
@@ -12903,7 +12941,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" ht="29.25">
       <c r="A19" s="240" t="s">
         <v>478</v>
       </c>
@@ -12947,7 +12985,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="15.75" thickBot="1">
+    <row r="23" spans="1:3">
       <c r="A23" s="240" t="s">
         <v>457</v>
       </c>
@@ -12959,11 +12997,11 @@
       </c>
     </row>
     <row r="24" spans="1:3">
-      <c r="A24" s="244" t="s">
+      <c r="A24" s="249" t="s">
         <v>490</v>
       </c>
-      <c r="B24" s="254"/>
-      <c r="C24" s="254"/>
+      <c r="B24" s="262"/>
+      <c r="C24" s="262"/>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="237" t="s">
@@ -13009,7 +13047,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15.75" thickBot="1">
+    <row r="29" spans="1:3">
       <c r="A29" s="237" t="s">
         <v>500</v>
       </c>
@@ -13021,13 +13059,13 @@
       </c>
     </row>
     <row r="30" spans="1:3">
-      <c r="A30" s="244" t="s">
+      <c r="A30" s="249" t="s">
         <v>503</v>
       </c>
-      <c r="B30" s="254"/>
-      <c r="C30" s="254"/>
-    </row>
-    <row r="31" spans="1:3">
+      <c r="B30" s="262"/>
+      <c r="C30" s="262"/>
+    </row>
+    <row r="31" spans="1:3" ht="29.25">
       <c r="A31" s="237" t="s">
         <v>504</v>
       </c>
@@ -13038,7 +13076,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" ht="29.25">
       <c r="A32" s="240" t="s">
         <v>507</v>
       </c>
@@ -13060,7 +13098,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="15.75" thickBot="1">
+    <row r="34" spans="1:3">
       <c r="A34" s="240" t="s">
         <v>500</v>
       </c>
@@ -13072,11 +13110,11 @@
       </c>
     </row>
     <row r="35" spans="1:3">
-      <c r="A35" s="244" t="s">
+      <c r="A35" s="249" t="s">
         <v>514</v>
       </c>
-      <c r="B35" s="254"/>
-      <c r="C35" s="254"/>
+      <c r="B35" s="262"/>
+      <c r="C35" s="262"/>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="237" t="s">
@@ -13122,7 +13160,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="15.75" thickBot="1">
+    <row r="40" spans="1:3">
       <c r="A40" s="237" t="s">
         <v>523</v>
       </c>
@@ -13134,13 +13172,13 @@
       </c>
     </row>
     <row r="41" spans="1:3">
-      <c r="A41" s="244" t="s">
+      <c r="A41" s="249" t="s">
         <v>525</v>
       </c>
-      <c r="B41" s="254"/>
-      <c r="C41" s="254"/>
-    </row>
-    <row r="42" spans="1:3">
+      <c r="B41" s="262"/>
+      <c r="C41" s="262"/>
+    </row>
+    <row r="42" spans="1:3" ht="29.25">
       <c r="A42" s="237" t="s">
         <v>478</v>
       </c>
@@ -13173,7 +13211,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="15.75" thickBot="1">
+    <row r="45" spans="1:3" ht="15.75">
       <c r="A45" s="240" t="s">
         <v>531</v>
       </c>
@@ -13185,13 +13223,13 @@
       </c>
     </row>
     <row r="46" spans="1:3">
-      <c r="A46" s="244" t="s">
+      <c r="A46" s="249" t="s">
         <v>534</v>
       </c>
-      <c r="B46" s="254"/>
-      <c r="C46" s="254"/>
-    </row>
-    <row r="47" spans="1:3">
+      <c r="B46" s="262"/>
+      <c r="C46" s="262"/>
+    </row>
+    <row r="47" spans="1:3" ht="29.25">
       <c r="A47" s="237" t="s">
         <v>515</v>
       </c>
@@ -13224,7 +13262,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="15.75" thickBot="1">
+    <row r="50" spans="1:3">
       <c r="A50" s="240" t="s">
         <v>500</v>
       </c>
@@ -13236,11 +13274,11 @@
       </c>
     </row>
     <row r="51" spans="1:3">
-      <c r="A51" s="244" t="s">
+      <c r="A51" s="249" t="s">
         <v>543</v>
       </c>
-      <c r="B51" s="254"/>
-      <c r="C51" s="254"/>
+      <c r="B51" s="262"/>
+      <c r="C51" s="262"/>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" s="237" t="s">
@@ -13304,23 +13342,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="8ee09cf5-53a8-4aeb-94af-927f54a7d6d8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005A4695005C4BEE4A8751FEE2C473E10D" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="df7fcaa21f93254d26451ff7a6d04ad2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="8ee09cf5-53a8-4aeb-94af-927f54a7d6d8" xmlns:ns4="ecf1487c-a58a-4bc0-a420-fb42a2a3dfc7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fefbcb393e90fe08e3723c038b505a33" ns3:_="" ns4:_="">
     <xsd:import namespace="8ee09cf5-53a8-4aeb-94af-927f54a7d6d8"/>
@@ -13559,14 +13580,31 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="8ee09cf5-53a8-4aeb-94af-927f54a7d6d8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A59486CE-8728-40BE-973B-B64C7CD06C40}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8E275EF-C000-4518-B0F8-FE9A60820B51}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC6EF48D-28DC-4A85-AE0A-77598A9ABE97}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A59486CE-8728-40BE-973B-B64C7CD06C40}"/>
 </file>
</xml_diff>

<commit_message>
Update app icon to sakura.jpg
</commit_message>
<xml_diff>
--- a/japantour.xlsx
+++ b/japantour.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bscvn-my.sharepoint.com/personal/minhpq_bsc_com_vn/Documents/09_CODER/00_travel-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="107" documentId="13_ncr:1_{4CBA3FCD-3F21-4F99-9320-E2DF1148D8FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B59818CB-455F-4711-86E1-8C5361AD4E42}"/>
+  <xr:revisionPtr revIDLastSave="165" documentId="13_ncr:1_{4CBA3FCD-3F21-4F99-9320-E2DF1148D8FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2B685CF-E5ED-4784-BE59-CD773F258209}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="458" firstSheet="4" activeTab="4" xr2:uid="{1D34A874-FA64-408A-8A73-D0DA492D543E}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="990" uniqueCount="562">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="571">
   <si>
     <t>Đơn giá</t>
   </si>
@@ -1403,10 +1403,7 @@
     <t>Send Luggage</t>
   </si>
   <si>
-    <t>Send Luggage at Yamato Transport</t>
-  </si>
-  <si>
-    <t>Yamato: Terminal 2, 3rd Floor</t>
+    <t>Yamato Transport on Terminal 2, 3rd Floor</t>
   </si>
   <si>
     <t>https://www.kuronekoyamato.co.jp/ytc/en/send/services/airport/narita2_send.html</t>
@@ -1418,10 +1415,10 @@
     <t>Airport Transfer</t>
   </si>
   <si>
-    <t>Transfer from Narita Airport to Tokyo via Keisei Skyliner / Train</t>
-  </si>
-  <si>
-    <t>Airbnb: 6-chōme-12-1 Ōmorikita エルメゾン大森203, Ota City, Tokyo</t>
+    <t>Transfer from Narita to Tokyo via Keisei Skyliner / Train</t>
+  </si>
+  <si>
+    <t>Airbnb</t>
   </si>
   <si>
     <t>https://maps.app.goo.gl/DBmdvffro3LetJej6</t>
@@ -1433,16 +1430,19 @@
     <t>Lunch</t>
   </si>
   <si>
-    <t>Enjoy authentic Japanese curry at CoCo Ichibanya.</t>
+    <t xml:space="preserve">Enjoy Japanese curry </t>
+  </si>
+  <si>
+    <t>CoCo Ichibanya</t>
   </si>
   <si>
     <t>13:00 - 14:00</t>
   </si>
   <si>
-    <t>Check-in &amp; Refresh</t>
-  </si>
-  <si>
-    <t>Airbnb Check in</t>
+    <t>Check-in</t>
+  </si>
+  <si>
+    <t>Airbnb Check in at 6-chōme-12-1 Ōmorikita エルメゾン大森203, Ota City, Tokyo</t>
   </si>
   <si>
     <t>14:00 - 16:30</t>
@@ -1451,7 +1451,13 @@
     <t>Miraikan Museum</t>
   </si>
   <si>
-    <t>Visit Miraikan (National Museum of Emerging Science and Innovation)</t>
+    <t>Visit National Museum of Emerging Science and Innovation</t>
+  </si>
+  <si>
+    <t>Miraikan</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/BmYZxEzfSyLjgQyp9</t>
   </si>
   <si>
     <t>16:30 - 17:30</t>
@@ -1460,7 +1466,13 @@
     <t>Odaiba Sunset</t>
   </si>
   <si>
-    <t>Sunset stroll at Odaiba Seaside Park; admire Rainbow Bridge and Tokyo Bay skyline.</t>
+    <t>Sunset stroll at Odaiba Seaside Park; Admire Rainbow Bridge and Tokyo Bay skyline.</t>
+  </si>
+  <si>
+    <t>Sunset point</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/t1SnqWYUNsLD9mvk7</t>
   </si>
   <si>
     <t>18:00 - 20:00</t>
@@ -1469,16 +1481,13 @@
     <t>Dinner</t>
   </si>
   <si>
-    <t>Traditional Tokyo Monjayaki specialty dinner</t>
-  </si>
-  <si>
-    <t>20:00 - 21:00</t>
-  </si>
-  <si>
-    <t>Evening Leisure</t>
-  </si>
-  <si>
-    <t>Night at Tokyo Tower and return hotel to rest</t>
+    <t>Traditional Tokyo Monjayaki dinner</t>
+  </si>
+  <si>
+    <t>Evening</t>
+  </si>
+  <si>
+    <t>Night at Tokyo and Return hotel to rest</t>
   </si>
   <si>
     <t xml:space="preserve">  Day 2: Tokyo DisneySea</t>
@@ -1490,28 +1499,31 @@
     <t>Transfer to Disney</t>
   </si>
   <si>
-    <t>Transfer from hotel to Tokyo DisneySea (Maihama, Chiba).</t>
+    <t>Transfer from hotel to Tokyo DisneySea</t>
+  </si>
+  <si>
+    <t>Tokyo DisneySea</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/mFXM4V9B9K4DBWVz8</t>
   </si>
   <si>
     <t>09:00 - 16:00</t>
   </si>
   <si>
-    <t>Tokyo DisneySea</t>
-  </si>
-  <si>
     <t>Full day exploring themed ports: Mediterranean Harbor, Mysterious Island, Arabian Coast &amp; thrilling attractions. Lunch inside park.</t>
   </si>
   <si>
     <t>17:00 - 21:00</t>
   </si>
   <si>
-    <t>Fresh kaiten-sushi dinner at Sushiro (Omorikita branch).</t>
-  </si>
-  <si>
-    <t>Return to Hotel</t>
-  </si>
-  <si>
-    <t>Evening leisure &amp; rest at hotel.</t>
+    <t>Fresh sushi dinner at Sushiro</t>
+  </si>
+  <si>
+    <t>Omorikita branch</t>
+  </si>
+  <si>
+    <t>https://share.google/glhiHLvLUNFKbIXOL</t>
   </si>
   <si>
     <t xml:space="preserve">  Day 3: Mount Fuji • Oshino Hakkai • Lake Kawaguchiko</t>
@@ -1523,7 +1535,7 @@
     <t>Depart for Mt. Fuji</t>
   </si>
   <si>
-    <t>Check out hotel; transfer from Tokyo toward Fuji Five Lakes region.</t>
+    <t>Check out hotel; Transfer from Tokyo toward Fuji Mount</t>
   </si>
   <si>
     <t>08:00 - 12:00</t>
@@ -1538,7 +1550,13 @@
     <t>12:00 - 13:30</t>
   </si>
   <si>
-    <t>Authentic Koshu Hoto Kosaku noodles (pumpkin miso noodle stew).</t>
+    <t>Authentic Koshu Hoto Kosaku noodles (Pumpkin miso noodle stew).</t>
+  </si>
+  <si>
+    <t>Huto Noodle</t>
+  </si>
+  <si>
+    <t>https://share.google/07foiHP82iKKrDXLN</t>
   </si>
   <si>
     <t>13:30 - 16:00</t>
@@ -1559,7 +1577,16 @@
     <t>Check in Fuji Kawaguchiko Resort Hotel; relax with Mount Fuji view.</t>
   </si>
   <si>
+    <t xml:space="preserve"> Fuji Kawaguchiko Resort Hotel</t>
+  </si>
+  <si>
+    <t>https://share.google/HkyzWgzwgKD1EYvWY</t>
+  </si>
+  <si>
     <t>Charcoal-grilled BBQ/ Yakitori dinner at Sanrokuen.</t>
+  </si>
+  <si>
+    <t>tiktok.com/@wethecurioustravelers/video/7350291288496901394?is_from_webapp=1&amp;sender_device=pc&amp;web_id=7410061434220971537</t>
   </si>
   <si>
     <t xml:space="preserve">  Day 4: Kawaguchiko • Matsumoto City</t>
@@ -2084,7 +2111,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -2147,74 +2174,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFD0D7DE"/>
+        <color theme="2"/>
       </left>
       <right style="thin">
-        <color rgb="FFD0D7DE"/>
+        <color theme="2"/>
       </right>
-      <top style="medium">
-        <color rgb="FF123056"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF123056"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD0D7DE"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD0D7DE"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF123056"/>
+      <top style="thin">
+        <color theme="2"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFD0D7DE"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD0D7DE"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD0D7DE"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD0D7DE"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD0D7DE"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD0D7DE"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD0D7DE"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD0D7DE"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD0D7DE"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD0D7DE"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFD0D7DE"/>
+        <color theme="2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -2224,7 +2193,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="274">
+  <cellXfs count="261">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2863,104 +2832,67 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="29" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="31" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="31" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="31" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="29" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="32" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="32" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
@@ -6036,7 +5968,7 @@
     <row r="137" spans="1:8" ht="15" customHeight="1">
       <c r="A137" s="37"/>
       <c r="B137" s="38"/>
-      <c r="C137" s="258" t="s">
+      <c r="C137" s="236" t="s">
         <v>179</v>
       </c>
       <c r="D137" s="38"/>
@@ -6051,7 +5983,7 @@
     <row r="138" spans="1:8" ht="15" customHeight="1">
       <c r="A138" s="37"/>
       <c r="B138" s="38"/>
-      <c r="C138" s="258"/>
+      <c r="C138" s="236"/>
       <c r="D138" s="38"/>
       <c r="E138" s="39"/>
       <c r="F138" s="38"/>
@@ -6777,8 +6709,8 @@
         <v>225</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="259" customFormat="1">
-      <c r="A2" s="259" t="s">
+    <row r="2" spans="1:10" s="237" customFormat="1">
+      <c r="A2" s="237" t="s">
         <v>226</v>
       </c>
     </row>
@@ -6885,10 +6817,10 @@
     <row r="8" spans="1:10">
       <c r="A8" s="84"/>
       <c r="B8" s="85"/>
-      <c r="C8" s="260" t="s">
+      <c r="C8" s="238" t="s">
         <v>230</v>
       </c>
-      <c r="D8" s="260"/>
+      <c r="D8" s="238"/>
       <c r="E8" s="96">
         <v>1500</v>
       </c>
@@ -6931,10 +6863,10 @@
       <c r="J10" s="85"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="260" t="s">
+      <c r="A11" s="238" t="s">
         <v>233</v>
       </c>
-      <c r="B11" s="260"/>
+      <c r="B11" s="238"/>
       <c r="C11" s="99">
         <v>27</v>
       </c>
@@ -9268,8 +9200,8 @@
         <v>225</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="259" customFormat="1">
-      <c r="A2" s="259" t="s">
+    <row r="2" spans="1:12" s="237" customFormat="1">
+      <c r="A2" s="237" t="s">
         <v>226</v>
       </c>
     </row>
@@ -9430,10 +9362,10 @@
     <row r="10" spans="1:12">
       <c r="A10" s="84"/>
       <c r="B10" s="85"/>
-      <c r="C10" s="260" t="s">
+      <c r="C10" s="238" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="260"/>
+      <c r="D10" s="238"/>
       <c r="E10" s="96">
         <v>3000</v>
       </c>
@@ -9476,10 +9408,10 @@
       <c r="J12" s="85"/>
     </row>
     <row r="13" spans="1:12">
-      <c r="A13" s="260" t="s">
+      <c r="A13" s="238" t="s">
         <v>233</v>
       </c>
-      <c r="B13" s="260"/>
+      <c r="B13" s="238"/>
       <c r="C13" s="99">
         <v>13</v>
       </c>
@@ -9903,10 +9835,10 @@
     <row r="34" spans="1:12">
       <c r="A34" s="114"/>
       <c r="B34" s="127"/>
-      <c r="C34" s="262" t="s">
+      <c r="C34" s="240" t="s">
         <v>338</v>
       </c>
-      <c r="D34" s="262"/>
+      <c r="D34" s="240"/>
       <c r="E34" s="128"/>
       <c r="F34" s="129"/>
       <c r="G34" s="127"/>
@@ -9919,10 +9851,10 @@
     <row r="35" spans="1:12">
       <c r="A35" s="114"/>
       <c r="B35" s="127"/>
-      <c r="C35" s="263" t="s">
+      <c r="C35" s="241" t="s">
         <v>50</v>
       </c>
-      <c r="D35" s="263"/>
+      <c r="D35" s="241"/>
       <c r="E35" s="128"/>
       <c r="F35" s="129"/>
       <c r="G35" s="127"/>
@@ -9939,10 +9871,10 @@
       <c r="B36" s="101">
         <v>0.33333333333333331</v>
       </c>
-      <c r="C36" s="265" t="s">
+      <c r="C36" s="243" t="s">
         <v>51</v>
       </c>
-      <c r="D36" s="265"/>
+      <c r="D36" s="243"/>
       <c r="E36" s="132"/>
       <c r="F36" s="133"/>
       <c r="G36" s="134"/>
@@ -10189,10 +10121,10 @@
     <row r="48" spans="1:12">
       <c r="A48" s="114"/>
       <c r="B48" s="109"/>
-      <c r="C48" s="264" t="s">
+      <c r="C48" s="242" t="s">
         <v>352</v>
       </c>
-      <c r="D48" s="264"/>
+      <c r="D48" s="242"/>
       <c r="E48" s="96">
         <f>370+220</f>
         <v>590</v>
@@ -10995,7 +10927,7 @@
     <row r="83" spans="1:10">
       <c r="A83" s="114"/>
       <c r="B83" s="109"/>
-      <c r="C83" s="261" t="s">
+      <c r="C83" s="239" t="s">
         <v>377</v>
       </c>
       <c r="D83" s="148" t="s">
@@ -11021,7 +10953,7 @@
     <row r="84" spans="1:10">
       <c r="A84" s="114"/>
       <c r="B84" s="109"/>
-      <c r="C84" s="261"/>
+      <c r="C84" s="239"/>
       <c r="D84" s="148" t="s">
         <v>379</v>
       </c>
@@ -12812,698 +12744,788 @@
     <col min="1" max="1" width="18" style="216" customWidth="1"/>
     <col min="2" max="2" width="28" style="216" customWidth="1"/>
     <col min="3" max="3" width="81" style="216" customWidth="1"/>
-    <col min="4" max="4" width="41.42578125" style="216" customWidth="1"/>
+    <col min="4" max="4" width="38" style="216" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.5703125" style="216" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="8.85546875" style="216"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="236" t="s">
+      <c r="A1" s="244" t="s">
         <v>432</v>
       </c>
-      <c r="B1" s="236" t="s">
+      <c r="B1" s="244" t="s">
         <v>433</v>
       </c>
-      <c r="C1" s="236" t="s">
+      <c r="C1" s="244" t="s">
         <v>434</v>
       </c>
-      <c r="D1" s="266" t="s">
+      <c r="D1" s="244" t="s">
         <v>435</v>
       </c>
-      <c r="E1" s="251" t="s">
+      <c r="E1" s="244" t="s">
         <v>436</v>
       </c>
-      <c r="F1" s="249" t="s">
+      <c r="F1" s="245" t="s">
         <v>437</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="256" t="s">
+      <c r="A2" s="246" t="s">
         <v>438</v>
       </c>
-      <c r="B2" s="271"/>
-      <c r="C2" s="271"/>
-      <c r="D2" s="267"/>
-      <c r="E2" s="252"/>
+      <c r="B2" s="259"/>
+      <c r="C2" s="259"/>
+      <c r="D2" s="247"/>
+      <c r="E2" s="247"/>
+      <c r="F2" s="248"/>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="237" t="s">
+      <c r="A3" s="249" t="s">
         <v>439</v>
       </c>
-      <c r="B3" s="238" t="s">
+      <c r="B3" s="250" t="s">
         <v>440</v>
       </c>
-      <c r="C3" s="239" t="s">
+      <c r="C3" s="251" t="s">
         <v>441</v>
       </c>
-      <c r="D3" s="268"/>
-      <c r="E3" s="253"/>
+      <c r="D3" s="251"/>
+      <c r="E3" s="251"/>
+      <c r="F3" s="248"/>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="240" t="s">
+      <c r="A4" s="252" t="s">
         <v>442</v>
       </c>
-      <c r="B4" s="241" t="s">
+      <c r="B4" s="253" t="s">
         <v>443</v>
       </c>
-      <c r="C4" s="242" t="s">
+      <c r="C4" s="254" t="s">
+        <v>443</v>
+      </c>
+      <c r="D4" s="254" t="s">
         <v>444</v>
       </c>
-      <c r="D4" s="269" t="s">
+      <c r="E4" s="254"/>
+      <c r="F4" s="255" t="s">
         <v>445</v>
       </c>
-      <c r="E4" s="254"/>
-      <c r="F4" s="8" t="s">
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="249" t="s">
         <v>446</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="30.75">
-      <c r="A5" s="237" t="s">
+      <c r="B5" s="250" t="s">
         <v>447</v>
       </c>
-      <c r="B5" s="238" t="s">
+      <c r="C5" s="251" t="s">
         <v>448</v>
       </c>
-      <c r="C5" s="239" t="s">
+      <c r="D5" s="251" t="s">
         <v>449</v>
       </c>
-      <c r="D5" s="268" t="s">
+      <c r="E5" s="251"/>
+      <c r="F5" s="256" t="s">
         <v>450</v>
       </c>
-      <c r="E5" s="253"/>
-      <c r="F5" s="250" t="s">
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="252" t="s">
         <v>451</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="240" t="s">
+      <c r="B6" s="253" t="s">
         <v>452</v>
       </c>
-      <c r="B6" s="241" t="s">
+      <c r="C6" s="254" t="s">
         <v>453</v>
       </c>
-      <c r="C6" s="242" t="s">
+      <c r="D6" s="254" t="s">
         <v>454</v>
       </c>
-      <c r="D6" s="269"/>
       <c r="E6" s="254"/>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="237" t="s">
+      <c r="F6" s="256" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.75">
+      <c r="A7" s="249" t="s">
         <v>455</v>
       </c>
-      <c r="B7" s="241" t="s">
+      <c r="B7" s="253" t="s">
         <v>456</v>
       </c>
-      <c r="C7" s="242" t="s">
+      <c r="C7" s="254" t="s">
         <v>457</v>
       </c>
-      <c r="D7" s="269"/>
+      <c r="D7" s="254"/>
       <c r="E7" s="254"/>
+      <c r="F7" s="248"/>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="240" t="s">
+      <c r="A8" s="252" t="s">
         <v>458</v>
       </c>
-      <c r="B8" s="241" t="s">
+      <c r="B8" s="253" t="s">
         <v>459</v>
       </c>
-      <c r="C8" s="242" t="s">
+      <c r="C8" s="254" t="s">
         <v>460</v>
       </c>
-      <c r="D8" s="269"/>
+      <c r="D8" s="254" t="s">
+        <v>461</v>
+      </c>
       <c r="E8" s="254"/>
+      <c r="F8" s="255" t="s">
+        <v>462</v>
+      </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="237" t="s">
-        <v>461</v>
-      </c>
-      <c r="B9" s="238" t="s">
-        <v>462</v>
-      </c>
-      <c r="C9" s="239" t="s">
+      <c r="A9" s="249" t="s">
         <v>463</v>
       </c>
-      <c r="D9" s="268"/>
-      <c r="E9" s="253"/>
+      <c r="B9" s="250" t="s">
+        <v>464</v>
+      </c>
+      <c r="C9" s="251" t="s">
+        <v>465</v>
+      </c>
+      <c r="D9" s="251" t="s">
+        <v>466</v>
+      </c>
+      <c r="E9" s="251"/>
+      <c r="F9" s="255" t="s">
+        <v>467</v>
+      </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="240" t="s">
-        <v>464</v>
-      </c>
-      <c r="B10" s="241" t="s">
-        <v>465</v>
-      </c>
-      <c r="C10" s="242" t="s">
-        <v>466</v>
-      </c>
-      <c r="D10" s="269"/>
+      <c r="A10" s="252" t="s">
+        <v>468</v>
+      </c>
+      <c r="B10" s="253" t="s">
+        <v>469</v>
+      </c>
+      <c r="C10" s="254" t="s">
+        <v>470</v>
+      </c>
+      <c r="D10" s="254"/>
       <c r="E10" s="254"/>
+      <c r="F10" s="248"/>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="243" t="s">
-        <v>467</v>
-      </c>
-      <c r="B11" s="244" t="s">
-        <v>468</v>
-      </c>
-      <c r="C11" s="245" t="s">
-        <v>469</v>
-      </c>
-      <c r="D11" s="268"/>
-      <c r="E11" s="253"/>
+      <c r="A11" s="258">
+        <v>0.875</v>
+      </c>
+      <c r="B11" s="250" t="s">
+        <v>471</v>
+      </c>
+      <c r="C11" s="251" t="s">
+        <v>472</v>
+      </c>
+      <c r="D11" s="251"/>
+      <c r="E11" s="251"/>
+      <c r="F11" s="248"/>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="257" t="s">
-        <v>470</v>
-      </c>
-      <c r="B12" s="272"/>
-      <c r="C12" s="272"/>
-      <c r="D12" s="270"/>
+        <v>473</v>
+      </c>
+      <c r="B12" s="260"/>
+      <c r="C12" s="260"/>
+      <c r="D12" s="248"/>
+      <c r="E12" s="248"/>
+      <c r="F12" s="248"/>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="237" t="s">
+      <c r="A13" s="249" t="s">
+        <v>474</v>
+      </c>
+      <c r="B13" s="250" t="s">
+        <v>475</v>
+      </c>
+      <c r="C13" s="251" t="s">
+        <v>476</v>
+      </c>
+      <c r="D13" s="251" t="s">
+        <v>477</v>
+      </c>
+      <c r="E13" s="251"/>
+      <c r="F13" s="255" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="29.25">
+      <c r="A14" s="252" t="s">
+        <v>479</v>
+      </c>
+      <c r="B14" s="253" t="s">
+        <v>477</v>
+      </c>
+      <c r="C14" s="254" t="s">
+        <v>480</v>
+      </c>
+      <c r="D14" s="254"/>
+      <c r="E14" s="254"/>
+      <c r="F14" s="248"/>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="249" t="s">
+        <v>481</v>
+      </c>
+      <c r="B15" s="250" t="s">
+        <v>469</v>
+      </c>
+      <c r="C15" s="251" t="s">
+        <v>482</v>
+      </c>
+      <c r="D15" s="251" t="s">
+        <v>483</v>
+      </c>
+      <c r="E15" s="251"/>
+      <c r="F15" s="255" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="258">
+        <v>0.875</v>
+      </c>
+      <c r="B16" s="250" t="s">
         <v>471</v>
       </c>
-      <c r="B13" s="238" t="s">
+      <c r="C16" s="251" t="s">
         <v>472</v>
       </c>
-      <c r="C13" s="239" t="s">
-        <v>473</v>
-      </c>
-      <c r="D13" s="268"/>
-      <c r="E13" s="253"/>
-    </row>
-    <row r="14" spans="1:6" ht="29.25">
-      <c r="A14" s="240" t="s">
-        <v>474</v>
-      </c>
-      <c r="B14" s="241" t="s">
-        <v>475</v>
-      </c>
-      <c r="C14" s="242" t="s">
-        <v>476</v>
-      </c>
-      <c r="D14" s="269"/>
-      <c r="E14" s="254"/>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" s="237" t="s">
-        <v>477</v>
-      </c>
-      <c r="B15" s="238" t="s">
-        <v>465</v>
-      </c>
-      <c r="C15" s="239" t="s">
-        <v>478</v>
-      </c>
-      <c r="D15" s="268"/>
-      <c r="E15" s="253"/>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" s="246">
-        <v>0.875</v>
-      </c>
-      <c r="B16" s="247" t="s">
-        <v>479</v>
-      </c>
-      <c r="C16" s="248" t="s">
-        <v>480</v>
-      </c>
-      <c r="D16" s="269"/>
+      <c r="D16" s="254"/>
       <c r="E16" s="254"/>
-    </row>
-    <row r="17" spans="1:5">
+      <c r="F16" s="248"/>
+    </row>
+    <row r="17" spans="1:6">
       <c r="A17" s="257" t="s">
-        <v>481</v>
-      </c>
-      <c r="B17" s="272"/>
-      <c r="C17" s="272"/>
-      <c r="D17" s="270"/>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="237" t="s">
-        <v>482</v>
-      </c>
-      <c r="B18" s="238" t="s">
-        <v>483</v>
-      </c>
-      <c r="C18" s="239" t="s">
-        <v>484</v>
-      </c>
-      <c r="D18" s="268"/>
-      <c r="E18" s="253"/>
-    </row>
-    <row r="19" spans="1:5" ht="29.25">
-      <c r="A19" s="240" t="s">
         <v>485</v>
       </c>
-      <c r="B19" s="241" t="s">
+      <c r="B17" s="260"/>
+      <c r="C17" s="260"/>
+      <c r="D17" s="248"/>
+      <c r="E17" s="248"/>
+      <c r="F17" s="248"/>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="249" t="s">
         <v>486</v>
       </c>
-      <c r="C19" s="242" t="s">
+      <c r="B18" s="250" t="s">
         <v>487</v>
       </c>
-      <c r="D19" s="269"/>
+      <c r="C18" s="251" t="s">
+        <v>488</v>
+      </c>
+      <c r="D18" s="251"/>
+      <c r="E18" s="251"/>
+      <c r="F18" s="248"/>
+    </row>
+    <row r="19" spans="1:6" ht="29.25">
+      <c r="A19" s="252" t="s">
+        <v>489</v>
+      </c>
+      <c r="B19" s="253" t="s">
+        <v>490</v>
+      </c>
+      <c r="C19" s="254" t="s">
+        <v>491</v>
+      </c>
+      <c r="D19" s="254"/>
       <c r="E19" s="254"/>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="237" t="s">
-        <v>488</v>
-      </c>
-      <c r="B20" s="238" t="s">
-        <v>453</v>
-      </c>
-      <c r="C20" s="239" t="s">
+      <c r="F19" s="248"/>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="249" t="s">
+        <v>492</v>
+      </c>
+      <c r="B20" s="250" t="s">
+        <v>452</v>
+      </c>
+      <c r="C20" s="251" t="s">
+        <v>493</v>
+      </c>
+      <c r="D20" s="251" t="s">
+        <v>494</v>
+      </c>
+      <c r="E20" s="251"/>
+      <c r="F20" s="255" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="252" t="s">
+        <v>496</v>
+      </c>
+      <c r="B21" s="253" t="s">
+        <v>497</v>
+      </c>
+      <c r="C21" s="254" t="s">
+        <v>498</v>
+      </c>
+      <c r="D21" s="254"/>
+      <c r="E21" s="254"/>
+      <c r="F21" s="248"/>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="249" t="s">
+        <v>499</v>
+      </c>
+      <c r="B22" s="250" t="s">
+        <v>500</v>
+      </c>
+      <c r="C22" s="251" t="s">
+        <v>501</v>
+      </c>
+      <c r="D22" s="251" t="s">
+        <v>502</v>
+      </c>
+      <c r="E22" s="251"/>
+      <c r="F22" s="255" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="252" t="s">
+        <v>468</v>
+      </c>
+      <c r="B23" s="253" t="s">
+        <v>469</v>
+      </c>
+      <c r="C23" s="254" t="s">
+        <v>504</v>
+      </c>
+      <c r="D23" s="254"/>
+      <c r="E23" s="254"/>
+      <c r="F23" s="8" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="257" t="s">
+        <v>506</v>
+      </c>
+      <c r="B24" s="260"/>
+      <c r="C24" s="260"/>
+      <c r="D24" s="248"/>
+      <c r="E24" s="248"/>
+      <c r="F24" s="248"/>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" s="249" t="s">
+        <v>507</v>
+      </c>
+      <c r="B25" s="250" t="s">
+        <v>508</v>
+      </c>
+      <c r="C25" s="251" t="s">
+        <v>509</v>
+      </c>
+      <c r="D25" s="251"/>
+      <c r="E25" s="251"/>
+      <c r="F25" s="248"/>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" s="252" t="s">
+        <v>510</v>
+      </c>
+      <c r="B26" s="253" t="s">
+        <v>452</v>
+      </c>
+      <c r="C26" s="254" t="s">
+        <v>511</v>
+      </c>
+      <c r="D26" s="254"/>
+      <c r="E26" s="254"/>
+      <c r="F26" s="248"/>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" s="249" t="s">
+        <v>512</v>
+      </c>
+      <c r="B27" s="250" t="s">
+        <v>513</v>
+      </c>
+      <c r="C27" s="251" t="s">
+        <v>514</v>
+      </c>
+      <c r="D27" s="251"/>
+      <c r="E27" s="251"/>
+      <c r="F27" s="248"/>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="252" t="s">
+        <v>499</v>
+      </c>
+      <c r="B28" s="253" t="s">
+        <v>500</v>
+      </c>
+      <c r="C28" s="254" t="s">
+        <v>515</v>
+      </c>
+      <c r="D28" s="254"/>
+      <c r="E28" s="254"/>
+      <c r="F28" s="248"/>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" s="249" t="s">
+        <v>516</v>
+      </c>
+      <c r="B29" s="250" t="s">
+        <v>517</v>
+      </c>
+      <c r="C29" s="251" t="s">
+        <v>518</v>
+      </c>
+      <c r="D29" s="251"/>
+      <c r="E29" s="251"/>
+      <c r="F29" s="248"/>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" s="257" t="s">
+        <v>519</v>
+      </c>
+      <c r="B30" s="260"/>
+      <c r="C30" s="260"/>
+      <c r="D30" s="248"/>
+      <c r="E30" s="248"/>
+      <c r="F30" s="248"/>
+    </row>
+    <row r="31" spans="1:6" ht="29.25">
+      <c r="A31" s="249" t="s">
+        <v>520</v>
+      </c>
+      <c r="B31" s="250" t="s">
+        <v>521</v>
+      </c>
+      <c r="C31" s="251" t="s">
+        <v>522</v>
+      </c>
+      <c r="D31" s="251"/>
+      <c r="E31" s="251"/>
+      <c r="F31" s="248"/>
+    </row>
+    <row r="32" spans="1:6" ht="29.25">
+      <c r="A32" s="252" t="s">
+        <v>523</v>
+      </c>
+      <c r="B32" s="253" t="s">
+        <v>524</v>
+      </c>
+      <c r="C32" s="254" t="s">
+        <v>525</v>
+      </c>
+      <c r="D32" s="254"/>
+      <c r="E32" s="254"/>
+      <c r="F32" s="248"/>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" s="249" t="s">
+        <v>526</v>
+      </c>
+      <c r="B33" s="250" t="s">
+        <v>527</v>
+      </c>
+      <c r="C33" s="251" t="s">
+        <v>528</v>
+      </c>
+      <c r="D33" s="251"/>
+      <c r="E33" s="251"/>
+      <c r="F33" s="248"/>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" s="252" t="s">
+        <v>516</v>
+      </c>
+      <c r="B34" s="253" t="s">
+        <v>469</v>
+      </c>
+      <c r="C34" s="254" t="s">
+        <v>529</v>
+      </c>
+      <c r="D34" s="254"/>
+      <c r="E34" s="254"/>
+      <c r="F34" s="248"/>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" s="257" t="s">
+        <v>530</v>
+      </c>
+      <c r="B35" s="260"/>
+      <c r="C35" s="260"/>
+      <c r="D35" s="248"/>
+      <c r="E35" s="248"/>
+      <c r="F35" s="248"/>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" s="249" t="s">
+        <v>531</v>
+      </c>
+      <c r="B36" s="250" t="s">
+        <v>532</v>
+      </c>
+      <c r="C36" s="251" t="s">
+        <v>533</v>
+      </c>
+      <c r="D36" s="251"/>
+      <c r="E36" s="251"/>
+      <c r="F36" s="248"/>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" s="252" t="s">
+        <v>510</v>
+      </c>
+      <c r="B37" s="253" t="s">
+        <v>452</v>
+      </c>
+      <c r="C37" s="254" t="s">
+        <v>534</v>
+      </c>
+      <c r="D37" s="254"/>
+      <c r="E37" s="254"/>
+      <c r="F37" s="248"/>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" s="249" t="s">
+        <v>512</v>
+      </c>
+      <c r="B38" s="250" t="s">
+        <v>535</v>
+      </c>
+      <c r="C38" s="251" t="s">
+        <v>536</v>
+      </c>
+      <c r="D38" s="251"/>
+      <c r="E38" s="251"/>
+      <c r="F38" s="248"/>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" s="252" t="s">
+        <v>537</v>
+      </c>
+      <c r="B39" s="253" t="s">
+        <v>500</v>
+      </c>
+      <c r="C39" s="254" t="s">
+        <v>538</v>
+      </c>
+      <c r="D39" s="254"/>
+      <c r="E39" s="254"/>
+      <c r="F39" s="248"/>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" s="249" t="s">
+        <v>539</v>
+      </c>
+      <c r="B40" s="250" t="s">
+        <v>469</v>
+      </c>
+      <c r="C40" s="251" t="s">
+        <v>540</v>
+      </c>
+      <c r="D40" s="251"/>
+      <c r="E40" s="251"/>
+      <c r="F40" s="248"/>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" s="257" t="s">
+        <v>541</v>
+      </c>
+      <c r="B41" s="260"/>
+      <c r="C41" s="260"/>
+      <c r="D41" s="248"/>
+      <c r="E41" s="248"/>
+      <c r="F41" s="248"/>
+    </row>
+    <row r="42" spans="1:6" ht="29.25">
+      <c r="A42" s="249" t="s">
         <v>489</v>
       </c>
-      <c r="D20" s="268"/>
-      <c r="E20" s="253"/>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" s="240" t="s">
-        <v>490</v>
-      </c>
-      <c r="B21" s="241" t="s">
-        <v>491</v>
-      </c>
-      <c r="C21" s="242" t="s">
+      <c r="B42" s="250" t="s">
+        <v>542</v>
+      </c>
+      <c r="C42" s="251" t="s">
+        <v>543</v>
+      </c>
+      <c r="D42" s="251"/>
+      <c r="E42" s="251"/>
+      <c r="F42" s="248"/>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" s="252" t="s">
         <v>492</v>
       </c>
-      <c r="D21" s="269"/>
-      <c r="E21" s="254"/>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" s="237" t="s">
-        <v>493</v>
-      </c>
-      <c r="B22" s="238" t="s">
-        <v>494</v>
-      </c>
-      <c r="C22" s="239" t="s">
-        <v>495</v>
-      </c>
-      <c r="D22" s="268"/>
-      <c r="E22" s="253"/>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" s="240" t="s">
-        <v>464</v>
-      </c>
-      <c r="B23" s="241" t="s">
-        <v>465</v>
-      </c>
-      <c r="C23" s="242" t="s">
-        <v>496</v>
-      </c>
-      <c r="D23" s="269"/>
-      <c r="E23" s="254"/>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" s="255" t="s">
-        <v>497</v>
-      </c>
-      <c r="B24" s="273"/>
-      <c r="C24" s="273"/>
-      <c r="D24" s="270"/>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" s="237" t="s">
-        <v>498</v>
-      </c>
-      <c r="B25" s="238" t="s">
-        <v>499</v>
-      </c>
-      <c r="C25" s="239" t="s">
-        <v>500</v>
-      </c>
-      <c r="D25" s="268"/>
-      <c r="E25" s="253"/>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" s="240" t="s">
-        <v>501</v>
-      </c>
-      <c r="B26" s="241" t="s">
-        <v>453</v>
-      </c>
-      <c r="C26" s="242" t="s">
-        <v>502</v>
-      </c>
-      <c r="D26" s="269"/>
-      <c r="E26" s="254"/>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" s="237" t="s">
-        <v>503</v>
-      </c>
-      <c r="B27" s="238" t="s">
-        <v>504</v>
-      </c>
-      <c r="C27" s="239" t="s">
-        <v>505</v>
-      </c>
-      <c r="D27" s="268"/>
-      <c r="E27" s="253"/>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" s="240" t="s">
-        <v>493</v>
-      </c>
-      <c r="B28" s="241" t="s">
-        <v>494</v>
-      </c>
-      <c r="C28" s="242" t="s">
-        <v>506</v>
-      </c>
-      <c r="D28" s="269"/>
-      <c r="E28" s="254"/>
-    </row>
-    <row r="29" spans="1:5">
-      <c r="A29" s="237" t="s">
-        <v>507</v>
-      </c>
-      <c r="B29" s="238" t="s">
-        <v>508</v>
-      </c>
-      <c r="C29" s="239" t="s">
-        <v>509</v>
-      </c>
-      <c r="D29" s="268"/>
-      <c r="E29" s="253"/>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" s="255" t="s">
+      <c r="B43" s="253" t="s">
+        <v>452</v>
+      </c>
+      <c r="C43" s="254" t="s">
+        <v>544</v>
+      </c>
+      <c r="D43" s="254"/>
+      <c r="E43" s="254"/>
+      <c r="F43" s="248"/>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" s="249" t="s">
+        <v>512</v>
+      </c>
+      <c r="B44" s="250" t="s">
+        <v>545</v>
+      </c>
+      <c r="C44" s="251" t="s">
+        <v>546</v>
+      </c>
+      <c r="D44" s="251"/>
+      <c r="E44" s="251"/>
+      <c r="F44" s="248"/>
+    </row>
+    <row r="45" spans="1:6" ht="15.75">
+      <c r="A45" s="252" t="s">
+        <v>547</v>
+      </c>
+      <c r="B45" s="253" t="s">
+        <v>548</v>
+      </c>
+      <c r="C45" s="254" t="s">
+        <v>549</v>
+      </c>
+      <c r="D45" s="254"/>
+      <c r="E45" s="254"/>
+      <c r="F45" s="248"/>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" s="257" t="s">
+        <v>550</v>
+      </c>
+      <c r="B46" s="260"/>
+      <c r="C46" s="260"/>
+      <c r="D46" s="248"/>
+      <c r="E46" s="248"/>
+      <c r="F46" s="248"/>
+    </row>
+    <row r="47" spans="1:6" ht="29.25">
+      <c r="A47" s="249" t="s">
+        <v>531</v>
+      </c>
+      <c r="B47" s="250" t="s">
+        <v>551</v>
+      </c>
+      <c r="C47" s="251" t="s">
+        <v>552</v>
+      </c>
+      <c r="D47" s="251"/>
+      <c r="E47" s="251"/>
+      <c r="F47" s="248"/>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48" s="252" t="s">
         <v>510</v>
       </c>
-      <c r="B30" s="273"/>
-      <c r="C30" s="273"/>
-      <c r="D30" s="270"/>
-    </row>
-    <row r="31" spans="1:5" ht="29.25">
-      <c r="A31" s="237" t="s">
-        <v>511</v>
-      </c>
-      <c r="B31" s="238" t="s">
-        <v>512</v>
-      </c>
-      <c r="C31" s="239" t="s">
-        <v>513</v>
-      </c>
-      <c r="D31" s="268"/>
-      <c r="E31" s="253"/>
-    </row>
-    <row r="32" spans="1:5" ht="29.25">
-      <c r="A32" s="240" t="s">
-        <v>514</v>
-      </c>
-      <c r="B32" s="241" t="s">
-        <v>515</v>
-      </c>
-      <c r="C32" s="242" t="s">
+      <c r="B48" s="253" t="s">
+        <v>452</v>
+      </c>
+      <c r="C48" s="254" t="s">
+        <v>553</v>
+      </c>
+      <c r="D48" s="254"/>
+      <c r="E48" s="254"/>
+      <c r="F48" s="248"/>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" s="249" t="s">
+        <v>554</v>
+      </c>
+      <c r="B49" s="250" t="s">
+        <v>555</v>
+      </c>
+      <c r="C49" s="251" t="s">
+        <v>556</v>
+      </c>
+      <c r="D49" s="251"/>
+      <c r="E49" s="251"/>
+      <c r="F49" s="248"/>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50" s="252" t="s">
         <v>516</v>
       </c>
-      <c r="D32" s="269"/>
-      <c r="E32" s="254"/>
-    </row>
-    <row r="33" spans="1:5">
-      <c r="A33" s="237" t="s">
-        <v>517</v>
-      </c>
-      <c r="B33" s="238" t="s">
-        <v>518</v>
-      </c>
-      <c r="C33" s="239" t="s">
-        <v>519</v>
-      </c>
-      <c r="D33" s="268"/>
-      <c r="E33" s="253"/>
-    </row>
-    <row r="34" spans="1:5">
-      <c r="A34" s="240" t="s">
-        <v>507</v>
-      </c>
-      <c r="B34" s="241" t="s">
-        <v>465</v>
-      </c>
-      <c r="C34" s="242" t="s">
-        <v>520</v>
-      </c>
-      <c r="D34" s="269"/>
-      <c r="E34" s="254"/>
-    </row>
-    <row r="35" spans="1:5">
-      <c r="A35" s="255" t="s">
-        <v>521</v>
-      </c>
-      <c r="B35" s="273"/>
-      <c r="C35" s="273"/>
-      <c r="D35" s="270"/>
-    </row>
-    <row r="36" spans="1:5">
-      <c r="A36" s="237" t="s">
-        <v>522</v>
-      </c>
-      <c r="B36" s="238" t="s">
-        <v>523</v>
-      </c>
-      <c r="C36" s="239" t="s">
-        <v>524</v>
-      </c>
-      <c r="D36" s="268"/>
-      <c r="E36" s="253"/>
-    </row>
-    <row r="37" spans="1:5">
-      <c r="A37" s="240" t="s">
-        <v>501</v>
-      </c>
-      <c r="B37" s="241" t="s">
-        <v>453</v>
-      </c>
-      <c r="C37" s="242" t="s">
-        <v>525</v>
-      </c>
-      <c r="D37" s="269"/>
-      <c r="E37" s="254"/>
-    </row>
-    <row r="38" spans="1:5">
-      <c r="A38" s="237" t="s">
-        <v>503</v>
-      </c>
-      <c r="B38" s="238" t="s">
-        <v>526</v>
-      </c>
-      <c r="C38" s="239" t="s">
-        <v>527</v>
-      </c>
-      <c r="D38" s="268"/>
-      <c r="E38" s="253"/>
-    </row>
-    <row r="39" spans="1:5">
-      <c r="A39" s="240" t="s">
-        <v>528</v>
-      </c>
-      <c r="B39" s="241" t="s">
-        <v>494</v>
-      </c>
-      <c r="C39" s="242" t="s">
-        <v>529</v>
-      </c>
-      <c r="D39" s="269"/>
-      <c r="E39" s="254"/>
-    </row>
-    <row r="40" spans="1:5">
-      <c r="A40" s="237" t="s">
-        <v>530</v>
-      </c>
-      <c r="B40" s="238" t="s">
-        <v>465</v>
-      </c>
-      <c r="C40" s="239" t="s">
-        <v>531</v>
-      </c>
-      <c r="D40" s="268"/>
-      <c r="E40" s="253"/>
-    </row>
-    <row r="41" spans="1:5">
-      <c r="A41" s="255" t="s">
-        <v>532</v>
-      </c>
-      <c r="B41" s="273"/>
-      <c r="C41" s="273"/>
-      <c r="D41" s="270"/>
-    </row>
-    <row r="42" spans="1:5" ht="29.25">
-      <c r="A42" s="237" t="s">
-        <v>485</v>
-      </c>
-      <c r="B42" s="238" t="s">
-        <v>533</v>
-      </c>
-      <c r="C42" s="239" t="s">
-        <v>534</v>
-      </c>
-      <c r="D42" s="268"/>
-      <c r="E42" s="253"/>
-    </row>
-    <row r="43" spans="1:5">
-      <c r="A43" s="240" t="s">
-        <v>488</v>
-      </c>
-      <c r="B43" s="241" t="s">
-        <v>453</v>
-      </c>
-      <c r="C43" s="242" t="s">
-        <v>535</v>
-      </c>
-      <c r="D43" s="269"/>
-      <c r="E43" s="254"/>
-    </row>
-    <row r="44" spans="1:5">
-      <c r="A44" s="237" t="s">
-        <v>503</v>
-      </c>
-      <c r="B44" s="238" t="s">
-        <v>536</v>
-      </c>
-      <c r="C44" s="239" t="s">
-        <v>537</v>
-      </c>
-      <c r="D44" s="268"/>
-      <c r="E44" s="253"/>
-    </row>
-    <row r="45" spans="1:5" ht="15.75">
-      <c r="A45" s="240" t="s">
-        <v>538</v>
-      </c>
-      <c r="B45" s="241" t="s">
-        <v>539</v>
-      </c>
-      <c r="C45" s="242" t="s">
-        <v>540</v>
-      </c>
-      <c r="D45" s="269"/>
-      <c r="E45" s="254"/>
-    </row>
-    <row r="46" spans="1:5">
-      <c r="A46" s="255" t="s">
-        <v>541</v>
-      </c>
-      <c r="B46" s="273"/>
-      <c r="C46" s="273"/>
-      <c r="D46" s="270"/>
-    </row>
-    <row r="47" spans="1:5" ht="29.25">
-      <c r="A47" s="237" t="s">
-        <v>522</v>
-      </c>
-      <c r="B47" s="238" t="s">
-        <v>542</v>
-      </c>
-      <c r="C47" s="239" t="s">
-        <v>543</v>
-      </c>
-      <c r="D47" s="268"/>
-      <c r="E47" s="253"/>
-    </row>
-    <row r="48" spans="1:5">
-      <c r="A48" s="240" t="s">
-        <v>501</v>
-      </c>
-      <c r="B48" s="241" t="s">
-        <v>453</v>
-      </c>
-      <c r="C48" s="242" t="s">
-        <v>544</v>
-      </c>
-      <c r="D48" s="269"/>
-      <c r="E48" s="254"/>
-    </row>
-    <row r="49" spans="1:5">
-      <c r="A49" s="237" t="s">
-        <v>545</v>
-      </c>
-      <c r="B49" s="238" t="s">
-        <v>546</v>
-      </c>
-      <c r="C49" s="239" t="s">
-        <v>547</v>
-      </c>
-      <c r="D49" s="268"/>
-      <c r="E49" s="253"/>
-    </row>
-    <row r="50" spans="1:5">
-      <c r="A50" s="240" t="s">
-        <v>507</v>
-      </c>
-      <c r="B50" s="241" t="s">
-        <v>548</v>
-      </c>
-      <c r="C50" s="242" t="s">
-        <v>549</v>
-      </c>
-      <c r="D50" s="269"/>
+      <c r="B50" s="253" t="s">
+        <v>557</v>
+      </c>
+      <c r="C50" s="254" t="s">
+        <v>558</v>
+      </c>
+      <c r="D50" s="254"/>
       <c r="E50" s="254"/>
-    </row>
-    <row r="51" spans="1:5">
-      <c r="A51" s="255" t="s">
-        <v>550</v>
-      </c>
-      <c r="B51" s="273"/>
-      <c r="C51" s="273"/>
-      <c r="D51" s="270"/>
-    </row>
-    <row r="52" spans="1:5">
-      <c r="A52" s="237" t="s">
-        <v>551</v>
-      </c>
-      <c r="B52" s="238" t="s">
-        <v>552</v>
-      </c>
-      <c r="C52" s="239" t="s">
-        <v>553</v>
-      </c>
-      <c r="D52" s="268"/>
-      <c r="E52" s="253"/>
-    </row>
-    <row r="53" spans="1:5">
-      <c r="A53" s="240" t="s">
-        <v>554</v>
-      </c>
-      <c r="B53" s="241" t="s">
-        <v>453</v>
-      </c>
-      <c r="C53" s="242" t="s">
-        <v>555</v>
-      </c>
-      <c r="D53" s="269"/>
+      <c r="F50" s="248"/>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" s="257" t="s">
+        <v>559</v>
+      </c>
+      <c r="B51" s="260"/>
+      <c r="C51" s="260"/>
+      <c r="D51" s="248"/>
+      <c r="E51" s="248"/>
+      <c r="F51" s="248"/>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" s="249" t="s">
+        <v>560</v>
+      </c>
+      <c r="B52" s="250" t="s">
+        <v>561</v>
+      </c>
+      <c r="C52" s="251" t="s">
+        <v>562</v>
+      </c>
+      <c r="D52" s="251"/>
+      <c r="E52" s="251"/>
+      <c r="F52" s="248"/>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53" s="252" t="s">
+        <v>563</v>
+      </c>
+      <c r="B53" s="253" t="s">
+        <v>452</v>
+      </c>
+      <c r="C53" s="254" t="s">
+        <v>564</v>
+      </c>
+      <c r="D53" s="254"/>
       <c r="E53" s="254"/>
-    </row>
-    <row r="54" spans="1:5">
-      <c r="A54" s="237" t="s">
-        <v>556</v>
-      </c>
-      <c r="B54" s="238" t="s">
-        <v>557</v>
-      </c>
-      <c r="C54" s="239" t="s">
-        <v>558</v>
-      </c>
-      <c r="D54" s="268"/>
-      <c r="E54" s="253"/>
-    </row>
-    <row r="55" spans="1:5">
-      <c r="A55" s="240" t="s">
-        <v>559</v>
-      </c>
-      <c r="B55" s="241" t="s">
-        <v>560</v>
-      </c>
-      <c r="C55" s="242" t="s">
-        <v>561</v>
-      </c>
-      <c r="D55" s="269"/>
+      <c r="F53" s="248"/>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" s="249" t="s">
+        <v>565</v>
+      </c>
+      <c r="B54" s="250" t="s">
+        <v>566</v>
+      </c>
+      <c r="C54" s="251" t="s">
+        <v>567</v>
+      </c>
+      <c r="D54" s="251"/>
+      <c r="E54" s="251"/>
+      <c r="F54" s="248"/>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" s="252" t="s">
+        <v>568</v>
+      </c>
+      <c r="B55" s="253" t="s">
+        <v>569</v>
+      </c>
+      <c r="C55" s="254" t="s">
+        <v>570</v>
+      </c>
+      <c r="D55" s="254"/>
       <c r="E55" s="254"/>
+      <c r="F55" s="248"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -13519,9 +13541,16 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F4" r:id="rId1" xr:uid="{6D84B550-56D9-418A-9D1C-EC3261D9DE2C}"/>
+    <hyperlink ref="F8" r:id="rId2" xr:uid="{362D1549-C6B0-4DBA-AF53-F162C8958291}"/>
+    <hyperlink ref="F9" r:id="rId3" xr:uid="{ABA130E2-28CF-48C2-9144-36C703EF636A}"/>
+    <hyperlink ref="F13" r:id="rId4" xr:uid="{E5CCB325-1CF9-4D32-BBF7-BAFC64ADBA13}"/>
+    <hyperlink ref="F15" r:id="rId5" xr:uid="{E2214F55-DBDD-417E-89D1-CBE8A004BF1C}"/>
+    <hyperlink ref="F20" r:id="rId6" xr:uid="{83714BB7-E198-4AF2-9E3F-F0EB6C640209}"/>
+    <hyperlink ref="F22" r:id="rId7" xr:uid="{3D986609-D1AD-40CD-9D91-B61C2D40A5ED}"/>
+    <hyperlink ref="F23" r:id="rId8" xr:uid="{9191FE3F-DA50-42C9-A969-CB2607764014}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" r:id="rId2"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" r:id="rId9"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Set 16:9 1920x1080 crop for images
</commit_message>
<xml_diff>
--- a/japantour.xlsx
+++ b/japantour.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bscvn-my.sharepoint.com/personal/minhpq_bsc_com_vn/Documents/09_CODER/00_travel-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="165" documentId="13_ncr:1_{4CBA3FCD-3F21-4F99-9320-E2DF1148D8FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2B685CF-E5ED-4784-BE59-CD773F258209}"/>
+  <xr:revisionPtr revIDLastSave="167" documentId="13_ncr:1_{4CBA3FCD-3F21-4F99-9320-E2DF1148D8FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD04243F-370A-43DE-9081-B5FB59FFBFE7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="458" firstSheet="4" activeTab="4" xr2:uid="{1D34A874-FA64-408A-8A73-D0DA492D543E}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1005" uniqueCount="573">
   <si>
     <t>Đơn giá</t>
   </si>
@@ -1434,6 +1434,12 @@
   </si>
   <si>
     <t>CoCo Ichibanya</t>
+  </si>
+  <si>
+    <t>1_day1_curryhouse.png</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/QUZeFor2cqwbRkzj7</t>
   </si>
   <si>
     <t>13:00 - 14:00</t>
@@ -2832,37 +2838,10 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="30" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="28" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="31" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2885,11 +2864,38 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="20" fontId="31" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="31" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="30" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -5968,7 +5974,7 @@
     <row r="137" spans="1:8" ht="15" customHeight="1">
       <c r="A137" s="37"/>
       <c r="B137" s="38"/>
-      <c r="C137" s="236" t="s">
+      <c r="C137" s="251" t="s">
         <v>179</v>
       </c>
       <c r="D137" s="38"/>
@@ -5983,7 +5989,7 @@
     <row r="138" spans="1:8" ht="15" customHeight="1">
       <c r="A138" s="37"/>
       <c r="B138" s="38"/>
-      <c r="C138" s="236"/>
+      <c r="C138" s="251"/>
       <c r="D138" s="38"/>
       <c r="E138" s="39"/>
       <c r="F138" s="38"/>
@@ -6709,8 +6715,8 @@
         <v>225</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="237" customFormat="1">
-      <c r="A2" s="237" t="s">
+    <row r="2" spans="1:10" s="252" customFormat="1">
+      <c r="A2" s="252" t="s">
         <v>226</v>
       </c>
     </row>
@@ -6817,10 +6823,10 @@
     <row r="8" spans="1:10">
       <c r="A8" s="84"/>
       <c r="B8" s="85"/>
-      <c r="C8" s="238" t="s">
+      <c r="C8" s="253" t="s">
         <v>230</v>
       </c>
-      <c r="D8" s="238"/>
+      <c r="D8" s="253"/>
       <c r="E8" s="96">
         <v>1500</v>
       </c>
@@ -6863,10 +6869,10 @@
       <c r="J10" s="85"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="238" t="s">
+      <c r="A11" s="253" t="s">
         <v>233</v>
       </c>
-      <c r="B11" s="238"/>
+      <c r="B11" s="253"/>
       <c r="C11" s="99">
         <v>27</v>
       </c>
@@ -9200,8 +9206,8 @@
         <v>225</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="237" customFormat="1">
-      <c r="A2" s="237" t="s">
+    <row r="2" spans="1:12" s="252" customFormat="1">
+      <c r="A2" s="252" t="s">
         <v>226</v>
       </c>
     </row>
@@ -9362,10 +9368,10 @@
     <row r="10" spans="1:12">
       <c r="A10" s="84"/>
       <c r="B10" s="85"/>
-      <c r="C10" s="238" t="s">
+      <c r="C10" s="253" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="238"/>
+      <c r="D10" s="253"/>
       <c r="E10" s="96">
         <v>3000</v>
       </c>
@@ -9408,10 +9414,10 @@
       <c r="J12" s="85"/>
     </row>
     <row r="13" spans="1:12">
-      <c r="A13" s="238" t="s">
+      <c r="A13" s="253" t="s">
         <v>233</v>
       </c>
-      <c r="B13" s="238"/>
+      <c r="B13" s="253"/>
       <c r="C13" s="99">
         <v>13</v>
       </c>
@@ -9835,10 +9841,10 @@
     <row r="34" spans="1:12">
       <c r="A34" s="114"/>
       <c r="B34" s="127"/>
-      <c r="C34" s="240" t="s">
+      <c r="C34" s="255" t="s">
         <v>338</v>
       </c>
-      <c r="D34" s="240"/>
+      <c r="D34" s="255"/>
       <c r="E34" s="128"/>
       <c r="F34" s="129"/>
       <c r="G34" s="127"/>
@@ -9851,10 +9857,10 @@
     <row r="35" spans="1:12">
       <c r="A35" s="114"/>
       <c r="B35" s="127"/>
-      <c r="C35" s="241" t="s">
+      <c r="C35" s="256" t="s">
         <v>50</v>
       </c>
-      <c r="D35" s="241"/>
+      <c r="D35" s="256"/>
       <c r="E35" s="128"/>
       <c r="F35" s="129"/>
       <c r="G35" s="127"/>
@@ -9871,10 +9877,10 @@
       <c r="B36" s="101">
         <v>0.33333333333333331</v>
       </c>
-      <c r="C36" s="243" t="s">
+      <c r="C36" s="258" t="s">
         <v>51</v>
       </c>
-      <c r="D36" s="243"/>
+      <c r="D36" s="258"/>
       <c r="E36" s="132"/>
       <c r="F36" s="133"/>
       <c r="G36" s="134"/>
@@ -10121,10 +10127,10 @@
     <row r="48" spans="1:12">
       <c r="A48" s="114"/>
       <c r="B48" s="109"/>
-      <c r="C48" s="242" t="s">
+      <c r="C48" s="257" t="s">
         <v>352</v>
       </c>
-      <c r="D48" s="242"/>
+      <c r="D48" s="257"/>
       <c r="E48" s="96">
         <f>370+220</f>
         <v>590</v>
@@ -10927,7 +10933,7 @@
     <row r="83" spans="1:10">
       <c r="A83" s="114"/>
       <c r="B83" s="109"/>
-      <c r="C83" s="239" t="s">
+      <c r="C83" s="254" t="s">
         <v>377</v>
       </c>
       <c r="D83" s="148" t="s">
@@ -10953,7 +10959,7 @@
     <row r="84" spans="1:10">
       <c r="A84" s="114"/>
       <c r="B84" s="109"/>
-      <c r="C84" s="239"/>
+      <c r="C84" s="254"/>
       <c r="D84" s="148" t="s">
         <v>379</v>
       </c>
@@ -12750,782 +12756,784 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="244" t="s">
+      <c r="A1" s="236" t="s">
         <v>432</v>
       </c>
-      <c r="B1" s="244" t="s">
+      <c r="B1" s="236" t="s">
         <v>433</v>
       </c>
-      <c r="C1" s="244" t="s">
+      <c r="C1" s="236" t="s">
         <v>434</v>
       </c>
-      <c r="D1" s="244" t="s">
+      <c r="D1" s="236" t="s">
         <v>435</v>
       </c>
-      <c r="E1" s="244" t="s">
+      <c r="E1" s="236" t="s">
         <v>436</v>
       </c>
-      <c r="F1" s="245" t="s">
+      <c r="F1" s="237" t="s">
         <v>437</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="246" t="s">
+      <c r="A2" s="250" t="s">
         <v>438</v>
       </c>
       <c r="B2" s="259"/>
       <c r="C2" s="259"/>
-      <c r="D2" s="247"/>
-      <c r="E2" s="247"/>
-      <c r="F2" s="248"/>
+      <c r="D2" s="238"/>
+      <c r="E2" s="238"/>
+      <c r="F2" s="239"/>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="249" t="s">
+      <c r="A3" s="240" t="s">
         <v>439</v>
       </c>
-      <c r="B3" s="250" t="s">
+      <c r="B3" s="241" t="s">
         <v>440</v>
       </c>
-      <c r="C3" s="251" t="s">
+      <c r="C3" s="242" t="s">
         <v>441</v>
       </c>
-      <c r="D3" s="251"/>
-      <c r="E3" s="251"/>
-      <c r="F3" s="248"/>
+      <c r="D3" s="242"/>
+      <c r="E3" s="242"/>
+      <c r="F3" s="239"/>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="252" t="s">
+      <c r="A4" s="243" t="s">
         <v>442</v>
       </c>
-      <c r="B4" s="253" t="s">
+      <c r="B4" s="244" t="s">
         <v>443</v>
       </c>
-      <c r="C4" s="254" t="s">
+      <c r="C4" s="245" t="s">
         <v>443</v>
       </c>
-      <c r="D4" s="254" t="s">
+      <c r="D4" s="245" t="s">
         <v>444</v>
       </c>
-      <c r="E4" s="254"/>
-      <c r="F4" s="255" t="s">
+      <c r="E4" s="245"/>
+      <c r="F4" s="246" t="s">
         <v>445</v>
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="249" t="s">
+      <c r="A5" s="240" t="s">
         <v>446</v>
       </c>
-      <c r="B5" s="250" t="s">
+      <c r="B5" s="241" t="s">
         <v>447</v>
       </c>
-      <c r="C5" s="251" t="s">
+      <c r="C5" s="242" t="s">
         <v>448</v>
       </c>
-      <c r="D5" s="251" t="s">
+      <c r="D5" s="242" t="s">
         <v>449</v>
       </c>
-      <c r="E5" s="251"/>
-      <c r="F5" s="256" t="s">
+      <c r="E5" s="242"/>
+      <c r="F5" s="247" t="s">
         <v>450</v>
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="252" t="s">
+      <c r="A6" s="243" t="s">
         <v>451</v>
       </c>
-      <c r="B6" s="253" t="s">
+      <c r="B6" s="244" t="s">
         <v>452</v>
       </c>
-      <c r="C6" s="254" t="s">
+      <c r="C6" s="245" t="s">
         <v>453</v>
       </c>
-      <c r="D6" s="254" t="s">
+      <c r="D6" s="245" t="s">
         <v>454</v>
       </c>
-      <c r="E6" s="254"/>
-      <c r="F6" s="256" t="s">
-        <v>450</v>
+      <c r="E6" s="8" t="s">
+        <v>455</v>
+      </c>
+      <c r="F6" s="246" t="s">
+        <v>456</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.75">
-      <c r="A7" s="249" t="s">
-        <v>455</v>
-      </c>
-      <c r="B7" s="253" t="s">
-        <v>456</v>
-      </c>
-      <c r="C7" s="254" t="s">
+      <c r="A7" s="240" t="s">
         <v>457</v>
       </c>
-      <c r="D7" s="254"/>
-      <c r="E7" s="254"/>
-      <c r="F7" s="248"/>
+      <c r="B7" s="244" t="s">
+        <v>458</v>
+      </c>
+      <c r="C7" s="245" t="s">
+        <v>459</v>
+      </c>
+      <c r="D7" s="245"/>
+      <c r="E7" s="245"/>
+      <c r="F7" s="239"/>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="252" t="s">
-        <v>458</v>
-      </c>
-      <c r="B8" s="253" t="s">
-        <v>459</v>
-      </c>
-      <c r="C8" s="254" t="s">
+      <c r="A8" s="243" t="s">
         <v>460</v>
       </c>
-      <c r="D8" s="254" t="s">
+      <c r="B8" s="244" t="s">
         <v>461</v>
       </c>
-      <c r="E8" s="254"/>
-      <c r="F8" s="255" t="s">
+      <c r="C8" s="245" t="s">
         <v>462</v>
       </c>
+      <c r="D8" s="245" t="s">
+        <v>463</v>
+      </c>
+      <c r="E8" s="245"/>
+      <c r="F8" s="246" t="s">
+        <v>464</v>
+      </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="249" t="s">
-        <v>463</v>
-      </c>
-      <c r="B9" s="250" t="s">
-        <v>464</v>
-      </c>
-      <c r="C9" s="251" t="s">
+      <c r="A9" s="240" t="s">
         <v>465</v>
       </c>
-      <c r="D9" s="251" t="s">
+      <c r="B9" s="241" t="s">
         <v>466</v>
       </c>
-      <c r="E9" s="251"/>
-      <c r="F9" s="255" t="s">
+      <c r="C9" s="242" t="s">
         <v>467</v>
       </c>
+      <c r="D9" s="242" t="s">
+        <v>468</v>
+      </c>
+      <c r="E9" s="242"/>
+      <c r="F9" s="246" t="s">
+        <v>469</v>
+      </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="252" t="s">
-        <v>468</v>
-      </c>
-      <c r="B10" s="253" t="s">
-        <v>469</v>
-      </c>
-      <c r="C10" s="254" t="s">
+      <c r="A10" s="243" t="s">
         <v>470</v>
       </c>
-      <c r="D10" s="254"/>
-      <c r="E10" s="254"/>
-      <c r="F10" s="248"/>
+      <c r="B10" s="244" t="s">
+        <v>471</v>
+      </c>
+      <c r="C10" s="245" t="s">
+        <v>472</v>
+      </c>
+      <c r="D10" s="245"/>
+      <c r="E10" s="245"/>
+      <c r="F10" s="239"/>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="258">
+      <c r="A11" s="248">
         <v>0.875</v>
       </c>
-      <c r="B11" s="250" t="s">
-        <v>471</v>
-      </c>
-      <c r="C11" s="251" t="s">
-        <v>472</v>
-      </c>
-      <c r="D11" s="251"/>
-      <c r="E11" s="251"/>
-      <c r="F11" s="248"/>
+      <c r="B11" s="241" t="s">
+        <v>473</v>
+      </c>
+      <c r="C11" s="242" t="s">
+        <v>474</v>
+      </c>
+      <c r="D11" s="242"/>
+      <c r="E11" s="242"/>
+      <c r="F11" s="239"/>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="257" t="s">
-        <v>473</v>
+      <c r="A12" s="249" t="s">
+        <v>475</v>
       </c>
       <c r="B12" s="260"/>
       <c r="C12" s="260"/>
-      <c r="D12" s="248"/>
-      <c r="E12" s="248"/>
-      <c r="F12" s="248"/>
+      <c r="D12" s="239"/>
+      <c r="E12" s="239"/>
+      <c r="F12" s="239"/>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="249" t="s">
+      <c r="A13" s="240" t="s">
+        <v>476</v>
+      </c>
+      <c r="B13" s="241" t="s">
+        <v>477</v>
+      </c>
+      <c r="C13" s="242" t="s">
+        <v>478</v>
+      </c>
+      <c r="D13" s="242" t="s">
+        <v>479</v>
+      </c>
+      <c r="E13" s="242"/>
+      <c r="F13" s="246" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="29.25">
+      <c r="A14" s="243" t="s">
+        <v>481</v>
+      </c>
+      <c r="B14" s="244" t="s">
+        <v>479</v>
+      </c>
+      <c r="C14" s="245" t="s">
+        <v>482</v>
+      </c>
+      <c r="D14" s="245"/>
+      <c r="E14" s="245"/>
+      <c r="F14" s="239"/>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="240" t="s">
+        <v>483</v>
+      </c>
+      <c r="B15" s="241" t="s">
+        <v>471</v>
+      </c>
+      <c r="C15" s="242" t="s">
+        <v>484</v>
+      </c>
+      <c r="D15" s="242" t="s">
+        <v>485</v>
+      </c>
+      <c r="E15" s="242"/>
+      <c r="F15" s="246" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="248">
+        <v>0.875</v>
+      </c>
+      <c r="B16" s="241" t="s">
+        <v>473</v>
+      </c>
+      <c r="C16" s="242" t="s">
         <v>474</v>
       </c>
-      <c r="B13" s="250" t="s">
-        <v>475</v>
-      </c>
-      <c r="C13" s="251" t="s">
-        <v>476</v>
-      </c>
-      <c r="D13" s="251" t="s">
-        <v>477</v>
-      </c>
-      <c r="E13" s="251"/>
-      <c r="F13" s="255" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="29.25">
-      <c r="A14" s="252" t="s">
-        <v>479</v>
-      </c>
-      <c r="B14" s="253" t="s">
-        <v>477</v>
-      </c>
-      <c r="C14" s="254" t="s">
-        <v>480</v>
-      </c>
-      <c r="D14" s="254"/>
-      <c r="E14" s="254"/>
-      <c r="F14" s="248"/>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" s="249" t="s">
-        <v>481</v>
-      </c>
-      <c r="B15" s="250" t="s">
-        <v>469</v>
-      </c>
-      <c r="C15" s="251" t="s">
-        <v>482</v>
-      </c>
-      <c r="D15" s="251" t="s">
-        <v>483</v>
-      </c>
-      <c r="E15" s="251"/>
-      <c r="F15" s="255" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" s="258">
-        <v>0.875</v>
-      </c>
-      <c r="B16" s="250" t="s">
-        <v>471</v>
-      </c>
-      <c r="C16" s="251" t="s">
-        <v>472</v>
-      </c>
-      <c r="D16" s="254"/>
-      <c r="E16" s="254"/>
-      <c r="F16" s="248"/>
+      <c r="D16" s="245"/>
+      <c r="E16" s="245"/>
+      <c r="F16" s="239"/>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="257" t="s">
-        <v>485</v>
+      <c r="A17" s="249" t="s">
+        <v>487</v>
       </c>
       <c r="B17" s="260"/>
       <c r="C17" s="260"/>
-      <c r="D17" s="248"/>
-      <c r="E17" s="248"/>
-      <c r="F17" s="248"/>
+      <c r="D17" s="239"/>
+      <c r="E17" s="239"/>
+      <c r="F17" s="239"/>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="249" t="s">
-        <v>486</v>
-      </c>
-      <c r="B18" s="250" t="s">
-        <v>487</v>
-      </c>
-      <c r="C18" s="251" t="s">
+      <c r="A18" s="240" t="s">
         <v>488</v>
       </c>
-      <c r="D18" s="251"/>
-      <c r="E18" s="251"/>
-      <c r="F18" s="248"/>
+      <c r="B18" s="241" t="s">
+        <v>489</v>
+      </c>
+      <c r="C18" s="242" t="s">
+        <v>490</v>
+      </c>
+      <c r="D18" s="242"/>
+      <c r="E18" s="242"/>
+      <c r="F18" s="239"/>
     </row>
     <row r="19" spans="1:6" ht="29.25">
-      <c r="A19" s="252" t="s">
-        <v>489</v>
-      </c>
-      <c r="B19" s="253" t="s">
-        <v>490</v>
-      </c>
-      <c r="C19" s="254" t="s">
+      <c r="A19" s="243" t="s">
         <v>491</v>
       </c>
-      <c r="D19" s="254"/>
-      <c r="E19" s="254"/>
-      <c r="F19" s="248"/>
+      <c r="B19" s="244" t="s">
+        <v>492</v>
+      </c>
+      <c r="C19" s="245" t="s">
+        <v>493</v>
+      </c>
+      <c r="D19" s="245"/>
+      <c r="E19" s="245"/>
+      <c r="F19" s="239"/>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="249" t="s">
-        <v>492</v>
-      </c>
-      <c r="B20" s="250" t="s">
+      <c r="A20" s="240" t="s">
+        <v>494</v>
+      </c>
+      <c r="B20" s="241" t="s">
         <v>452</v>
       </c>
-      <c r="C20" s="251" t="s">
-        <v>493</v>
-      </c>
-      <c r="D20" s="251" t="s">
-        <v>494</v>
-      </c>
-      <c r="E20" s="251"/>
-      <c r="F20" s="255" t="s">
+      <c r="C20" s="242" t="s">
         <v>495</v>
       </c>
+      <c r="D20" s="242" t="s">
+        <v>496</v>
+      </c>
+      <c r="E20" s="242"/>
+      <c r="F20" s="246" t="s">
+        <v>497</v>
+      </c>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="252" t="s">
-        <v>496</v>
-      </c>
-      <c r="B21" s="253" t="s">
-        <v>497</v>
-      </c>
-      <c r="C21" s="254" t="s">
+      <c r="A21" s="243" t="s">
         <v>498</v>
       </c>
-      <c r="D21" s="254"/>
-      <c r="E21" s="254"/>
-      <c r="F21" s="248"/>
+      <c r="B21" s="244" t="s">
+        <v>499</v>
+      </c>
+      <c r="C21" s="245" t="s">
+        <v>500</v>
+      </c>
+      <c r="D21" s="245"/>
+      <c r="E21" s="245"/>
+      <c r="F21" s="239"/>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="249" t="s">
-        <v>499</v>
-      </c>
-      <c r="B22" s="250" t="s">
-        <v>500</v>
-      </c>
-      <c r="C22" s="251" t="s">
+      <c r="A22" s="240" t="s">
         <v>501</v>
       </c>
-      <c r="D22" s="251" t="s">
+      <c r="B22" s="241" t="s">
         <v>502</v>
       </c>
-      <c r="E22" s="251"/>
-      <c r="F22" s="255" t="s">
+      <c r="C22" s="242" t="s">
         <v>503</v>
       </c>
+      <c r="D22" s="242" t="s">
+        <v>504</v>
+      </c>
+      <c r="E22" s="242"/>
+      <c r="F22" s="246" t="s">
+        <v>505</v>
+      </c>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="252" t="s">
-        <v>468</v>
-      </c>
-      <c r="B23" s="253" t="s">
-        <v>469</v>
-      </c>
-      <c r="C23" s="254" t="s">
-        <v>504</v>
-      </c>
-      <c r="D23" s="254"/>
-      <c r="E23" s="254"/>
+      <c r="A23" s="243" t="s">
+        <v>470</v>
+      </c>
+      <c r="B23" s="244" t="s">
+        <v>471</v>
+      </c>
+      <c r="C23" s="245" t="s">
+        <v>506</v>
+      </c>
+      <c r="D23" s="245"/>
+      <c r="E23" s="245"/>
       <c r="F23" s="8" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="257" t="s">
-        <v>506</v>
+      <c r="A24" s="249" t="s">
+        <v>508</v>
       </c>
       <c r="B24" s="260"/>
       <c r="C24" s="260"/>
-      <c r="D24" s="248"/>
-      <c r="E24" s="248"/>
-      <c r="F24" s="248"/>
+      <c r="D24" s="239"/>
+      <c r="E24" s="239"/>
+      <c r="F24" s="239"/>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="249" t="s">
-        <v>507</v>
-      </c>
-      <c r="B25" s="250" t="s">
-        <v>508</v>
-      </c>
-      <c r="C25" s="251" t="s">
+      <c r="A25" s="240" t="s">
         <v>509</v>
       </c>
-      <c r="D25" s="251"/>
-      <c r="E25" s="251"/>
-      <c r="F25" s="248"/>
+      <c r="B25" s="241" t="s">
+        <v>510</v>
+      </c>
+      <c r="C25" s="242" t="s">
+        <v>511</v>
+      </c>
+      <c r="D25" s="242"/>
+      <c r="E25" s="242"/>
+      <c r="F25" s="239"/>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="252" t="s">
-        <v>510</v>
-      </c>
-      <c r="B26" s="253" t="s">
+      <c r="A26" s="243" t="s">
+        <v>512</v>
+      </c>
+      <c r="B26" s="244" t="s">
         <v>452</v>
       </c>
-      <c r="C26" s="254" t="s">
-        <v>511</v>
-      </c>
-      <c r="D26" s="254"/>
-      <c r="E26" s="254"/>
-      <c r="F26" s="248"/>
+      <c r="C26" s="245" t="s">
+        <v>513</v>
+      </c>
+      <c r="D26" s="245"/>
+      <c r="E26" s="245"/>
+      <c r="F26" s="239"/>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="249" t="s">
-        <v>512</v>
-      </c>
-      <c r="B27" s="250" t="s">
-        <v>513</v>
-      </c>
-      <c r="C27" s="251" t="s">
+      <c r="A27" s="240" t="s">
         <v>514</v>
       </c>
-      <c r="D27" s="251"/>
-      <c r="E27" s="251"/>
-      <c r="F27" s="248"/>
+      <c r="B27" s="241" t="s">
+        <v>515</v>
+      </c>
+      <c r="C27" s="242" t="s">
+        <v>516</v>
+      </c>
+      <c r="D27" s="242"/>
+      <c r="E27" s="242"/>
+      <c r="F27" s="239"/>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="252" t="s">
-        <v>499</v>
-      </c>
-      <c r="B28" s="253" t="s">
-        <v>500</v>
-      </c>
-      <c r="C28" s="254" t="s">
-        <v>515</v>
-      </c>
-      <c r="D28" s="254"/>
-      <c r="E28" s="254"/>
-      <c r="F28" s="248"/>
+      <c r="A28" s="243" t="s">
+        <v>501</v>
+      </c>
+      <c r="B28" s="244" t="s">
+        <v>502</v>
+      </c>
+      <c r="C28" s="245" t="s">
+        <v>517</v>
+      </c>
+      <c r="D28" s="245"/>
+      <c r="E28" s="245"/>
+      <c r="F28" s="239"/>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="249" t="s">
-        <v>516</v>
-      </c>
-      <c r="B29" s="250" t="s">
-        <v>517</v>
-      </c>
-      <c r="C29" s="251" t="s">
+      <c r="A29" s="240" t="s">
         <v>518</v>
       </c>
-      <c r="D29" s="251"/>
-      <c r="E29" s="251"/>
-      <c r="F29" s="248"/>
+      <c r="B29" s="241" t="s">
+        <v>519</v>
+      </c>
+      <c r="C29" s="242" t="s">
+        <v>520</v>
+      </c>
+      <c r="D29" s="242"/>
+      <c r="E29" s="242"/>
+      <c r="F29" s="239"/>
     </row>
     <row r="30" spans="1:6">
-      <c r="A30" s="257" t="s">
-        <v>519</v>
+      <c r="A30" s="249" t="s">
+        <v>521</v>
       </c>
       <c r="B30" s="260"/>
       <c r="C30" s="260"/>
-      <c r="D30" s="248"/>
-      <c r="E30" s="248"/>
-      <c r="F30" s="248"/>
+      <c r="D30" s="239"/>
+      <c r="E30" s="239"/>
+      <c r="F30" s="239"/>
     </row>
     <row r="31" spans="1:6" ht="29.25">
-      <c r="A31" s="249" t="s">
-        <v>520</v>
-      </c>
-      <c r="B31" s="250" t="s">
-        <v>521</v>
-      </c>
-      <c r="C31" s="251" t="s">
+      <c r="A31" s="240" t="s">
         <v>522</v>
       </c>
-      <c r="D31" s="251"/>
-      <c r="E31" s="251"/>
-      <c r="F31" s="248"/>
+      <c r="B31" s="241" t="s">
+        <v>523</v>
+      </c>
+      <c r="C31" s="242" t="s">
+        <v>524</v>
+      </c>
+      <c r="D31" s="242"/>
+      <c r="E31" s="242"/>
+      <c r="F31" s="239"/>
     </row>
     <row r="32" spans="1:6" ht="29.25">
-      <c r="A32" s="252" t="s">
-        <v>523</v>
-      </c>
-      <c r="B32" s="253" t="s">
-        <v>524</v>
-      </c>
-      <c r="C32" s="254" t="s">
+      <c r="A32" s="243" t="s">
         <v>525</v>
       </c>
-      <c r="D32" s="254"/>
-      <c r="E32" s="254"/>
-      <c r="F32" s="248"/>
+      <c r="B32" s="244" t="s">
+        <v>526</v>
+      </c>
+      <c r="C32" s="245" t="s">
+        <v>527</v>
+      </c>
+      <c r="D32" s="245"/>
+      <c r="E32" s="245"/>
+      <c r="F32" s="239"/>
     </row>
     <row r="33" spans="1:6">
-      <c r="A33" s="249" t="s">
-        <v>526</v>
-      </c>
-      <c r="B33" s="250" t="s">
-        <v>527</v>
-      </c>
-      <c r="C33" s="251" t="s">
+      <c r="A33" s="240" t="s">
         <v>528</v>
       </c>
-      <c r="D33" s="251"/>
-      <c r="E33" s="251"/>
-      <c r="F33" s="248"/>
+      <c r="B33" s="241" t="s">
+        <v>529</v>
+      </c>
+      <c r="C33" s="242" t="s">
+        <v>530</v>
+      </c>
+      <c r="D33" s="242"/>
+      <c r="E33" s="242"/>
+      <c r="F33" s="239"/>
     </row>
     <row r="34" spans="1:6">
-      <c r="A34" s="252" t="s">
-        <v>516</v>
-      </c>
-      <c r="B34" s="253" t="s">
-        <v>469</v>
-      </c>
-      <c r="C34" s="254" t="s">
-        <v>529</v>
-      </c>
-      <c r="D34" s="254"/>
-      <c r="E34" s="254"/>
-      <c r="F34" s="248"/>
+      <c r="A34" s="243" t="s">
+        <v>518</v>
+      </c>
+      <c r="B34" s="244" t="s">
+        <v>471</v>
+      </c>
+      <c r="C34" s="245" t="s">
+        <v>531</v>
+      </c>
+      <c r="D34" s="245"/>
+      <c r="E34" s="245"/>
+      <c r="F34" s="239"/>
     </row>
     <row r="35" spans="1:6">
-      <c r="A35" s="257" t="s">
-        <v>530</v>
+      <c r="A35" s="249" t="s">
+        <v>532</v>
       </c>
       <c r="B35" s="260"/>
       <c r="C35" s="260"/>
-      <c r="D35" s="248"/>
-      <c r="E35" s="248"/>
-      <c r="F35" s="248"/>
+      <c r="D35" s="239"/>
+      <c r="E35" s="239"/>
+      <c r="F35" s="239"/>
     </row>
     <row r="36" spans="1:6">
-      <c r="A36" s="249" t="s">
-        <v>531</v>
-      </c>
-      <c r="B36" s="250" t="s">
-        <v>532</v>
-      </c>
-      <c r="C36" s="251" t="s">
+      <c r="A36" s="240" t="s">
         <v>533</v>
       </c>
-      <c r="D36" s="251"/>
-      <c r="E36" s="251"/>
-      <c r="F36" s="248"/>
+      <c r="B36" s="241" t="s">
+        <v>534</v>
+      </c>
+      <c r="C36" s="242" t="s">
+        <v>535</v>
+      </c>
+      <c r="D36" s="242"/>
+      <c r="E36" s="242"/>
+      <c r="F36" s="239"/>
     </row>
     <row r="37" spans="1:6">
-      <c r="A37" s="252" t="s">
-        <v>510</v>
-      </c>
-      <c r="B37" s="253" t="s">
+      <c r="A37" s="243" t="s">
+        <v>512</v>
+      </c>
+      <c r="B37" s="244" t="s">
         <v>452</v>
       </c>
-      <c r="C37" s="254" t="s">
-        <v>534</v>
-      </c>
-      <c r="D37" s="254"/>
-      <c r="E37" s="254"/>
-      <c r="F37" s="248"/>
+      <c r="C37" s="245" t="s">
+        <v>536</v>
+      </c>
+      <c r="D37" s="245"/>
+      <c r="E37" s="245"/>
+      <c r="F37" s="239"/>
     </row>
     <row r="38" spans="1:6">
-      <c r="A38" s="249" t="s">
-        <v>512</v>
-      </c>
-      <c r="B38" s="250" t="s">
-        <v>535</v>
-      </c>
-      <c r="C38" s="251" t="s">
-        <v>536</v>
-      </c>
-      <c r="D38" s="251"/>
-      <c r="E38" s="251"/>
-      <c r="F38" s="248"/>
+      <c r="A38" s="240" t="s">
+        <v>514</v>
+      </c>
+      <c r="B38" s="241" t="s">
+        <v>537</v>
+      </c>
+      <c r="C38" s="242" t="s">
+        <v>538</v>
+      </c>
+      <c r="D38" s="242"/>
+      <c r="E38" s="242"/>
+      <c r="F38" s="239"/>
     </row>
     <row r="39" spans="1:6">
-      <c r="A39" s="252" t="s">
-        <v>537</v>
-      </c>
-      <c r="B39" s="253" t="s">
-        <v>500</v>
-      </c>
-      <c r="C39" s="254" t="s">
-        <v>538</v>
-      </c>
-      <c r="D39" s="254"/>
-      <c r="E39" s="254"/>
-      <c r="F39" s="248"/>
+      <c r="A39" s="243" t="s">
+        <v>539</v>
+      </c>
+      <c r="B39" s="244" t="s">
+        <v>502</v>
+      </c>
+      <c r="C39" s="245" t="s">
+        <v>540</v>
+      </c>
+      <c r="D39" s="245"/>
+      <c r="E39" s="245"/>
+      <c r="F39" s="239"/>
     </row>
     <row r="40" spans="1:6">
-      <c r="A40" s="249" t="s">
-        <v>539</v>
-      </c>
-      <c r="B40" s="250" t="s">
-        <v>469</v>
-      </c>
-      <c r="C40" s="251" t="s">
-        <v>540</v>
-      </c>
-      <c r="D40" s="251"/>
-      <c r="E40" s="251"/>
-      <c r="F40" s="248"/>
+      <c r="A40" s="240" t="s">
+        <v>541</v>
+      </c>
+      <c r="B40" s="241" t="s">
+        <v>471</v>
+      </c>
+      <c r="C40" s="242" t="s">
+        <v>542</v>
+      </c>
+      <c r="D40" s="242"/>
+      <c r="E40" s="242"/>
+      <c r="F40" s="239"/>
     </row>
     <row r="41" spans="1:6">
-      <c r="A41" s="257" t="s">
-        <v>541</v>
+      <c r="A41" s="249" t="s">
+        <v>543</v>
       </c>
       <c r="B41" s="260"/>
       <c r="C41" s="260"/>
-      <c r="D41" s="248"/>
-      <c r="E41" s="248"/>
-      <c r="F41" s="248"/>
+      <c r="D41" s="239"/>
+      <c r="E41" s="239"/>
+      <c r="F41" s="239"/>
     </row>
     <row r="42" spans="1:6" ht="29.25">
-      <c r="A42" s="249" t="s">
-        <v>489</v>
-      </c>
-      <c r="B42" s="250" t="s">
-        <v>542</v>
-      </c>
-      <c r="C42" s="251" t="s">
-        <v>543</v>
-      </c>
-      <c r="D42" s="251"/>
-      <c r="E42" s="251"/>
-      <c r="F42" s="248"/>
+      <c r="A42" s="240" t="s">
+        <v>491</v>
+      </c>
+      <c r="B42" s="241" t="s">
+        <v>544</v>
+      </c>
+      <c r="C42" s="242" t="s">
+        <v>545</v>
+      </c>
+      <c r="D42" s="242"/>
+      <c r="E42" s="242"/>
+      <c r="F42" s="239"/>
     </row>
     <row r="43" spans="1:6">
-      <c r="A43" s="252" t="s">
-        <v>492</v>
-      </c>
-      <c r="B43" s="253" t="s">
+      <c r="A43" s="243" t="s">
+        <v>494</v>
+      </c>
+      <c r="B43" s="244" t="s">
         <v>452</v>
       </c>
-      <c r="C43" s="254" t="s">
-        <v>544</v>
-      </c>
-      <c r="D43" s="254"/>
-      <c r="E43" s="254"/>
-      <c r="F43" s="248"/>
+      <c r="C43" s="245" t="s">
+        <v>546</v>
+      </c>
+      <c r="D43" s="245"/>
+      <c r="E43" s="245"/>
+      <c r="F43" s="239"/>
     </row>
     <row r="44" spans="1:6">
-      <c r="A44" s="249" t="s">
-        <v>512</v>
-      </c>
-      <c r="B44" s="250" t="s">
-        <v>545</v>
-      </c>
-      <c r="C44" s="251" t="s">
-        <v>546</v>
-      </c>
-      <c r="D44" s="251"/>
-      <c r="E44" s="251"/>
-      <c r="F44" s="248"/>
+      <c r="A44" s="240" t="s">
+        <v>514</v>
+      </c>
+      <c r="B44" s="241" t="s">
+        <v>547</v>
+      </c>
+      <c r="C44" s="242" t="s">
+        <v>548</v>
+      </c>
+      <c r="D44" s="242"/>
+      <c r="E44" s="242"/>
+      <c r="F44" s="239"/>
     </row>
     <row r="45" spans="1:6" ht="15.75">
-      <c r="A45" s="252" t="s">
-        <v>547</v>
-      </c>
-      <c r="B45" s="253" t="s">
-        <v>548</v>
-      </c>
-      <c r="C45" s="254" t="s">
+      <c r="A45" s="243" t="s">
         <v>549</v>
       </c>
-      <c r="D45" s="254"/>
-      <c r="E45" s="254"/>
-      <c r="F45" s="248"/>
+      <c r="B45" s="244" t="s">
+        <v>550</v>
+      </c>
+      <c r="C45" s="245" t="s">
+        <v>551</v>
+      </c>
+      <c r="D45" s="245"/>
+      <c r="E45" s="245"/>
+      <c r="F45" s="239"/>
     </row>
     <row r="46" spans="1:6">
-      <c r="A46" s="257" t="s">
-        <v>550</v>
+      <c r="A46" s="249" t="s">
+        <v>552</v>
       </c>
       <c r="B46" s="260"/>
       <c r="C46" s="260"/>
-      <c r="D46" s="248"/>
-      <c r="E46" s="248"/>
-      <c r="F46" s="248"/>
+      <c r="D46" s="239"/>
+      <c r="E46" s="239"/>
+      <c r="F46" s="239"/>
     </row>
     <row r="47" spans="1:6" ht="29.25">
-      <c r="A47" s="249" t="s">
-        <v>531</v>
-      </c>
-      <c r="B47" s="250" t="s">
-        <v>551</v>
-      </c>
-      <c r="C47" s="251" t="s">
-        <v>552</v>
-      </c>
-      <c r="D47" s="251"/>
-      <c r="E47" s="251"/>
-      <c r="F47" s="248"/>
+      <c r="A47" s="240" t="s">
+        <v>533</v>
+      </c>
+      <c r="B47" s="241" t="s">
+        <v>553</v>
+      </c>
+      <c r="C47" s="242" t="s">
+        <v>554</v>
+      </c>
+      <c r="D47" s="242"/>
+      <c r="E47" s="242"/>
+      <c r="F47" s="239"/>
     </row>
     <row r="48" spans="1:6">
-      <c r="A48" s="252" t="s">
-        <v>510</v>
-      </c>
-      <c r="B48" s="253" t="s">
+      <c r="A48" s="243" t="s">
+        <v>512</v>
+      </c>
+      <c r="B48" s="244" t="s">
         <v>452</v>
       </c>
-      <c r="C48" s="254" t="s">
-        <v>553</v>
-      </c>
-      <c r="D48" s="254"/>
-      <c r="E48" s="254"/>
-      <c r="F48" s="248"/>
+      <c r="C48" s="245" t="s">
+        <v>555</v>
+      </c>
+      <c r="D48" s="245"/>
+      <c r="E48" s="245"/>
+      <c r="F48" s="239"/>
     </row>
     <row r="49" spans="1:6">
-      <c r="A49" s="249" t="s">
-        <v>554</v>
-      </c>
-      <c r="B49" s="250" t="s">
-        <v>555</v>
-      </c>
-      <c r="C49" s="251" t="s">
+      <c r="A49" s="240" t="s">
         <v>556</v>
       </c>
-      <c r="D49" s="251"/>
-      <c r="E49" s="251"/>
-      <c r="F49" s="248"/>
+      <c r="B49" s="241" t="s">
+        <v>557</v>
+      </c>
+      <c r="C49" s="242" t="s">
+        <v>558</v>
+      </c>
+      <c r="D49" s="242"/>
+      <c r="E49" s="242"/>
+      <c r="F49" s="239"/>
     </row>
     <row r="50" spans="1:6">
-      <c r="A50" s="252" t="s">
-        <v>516</v>
-      </c>
-      <c r="B50" s="253" t="s">
-        <v>557</v>
-      </c>
-      <c r="C50" s="254" t="s">
-        <v>558</v>
-      </c>
-      <c r="D50" s="254"/>
-      <c r="E50" s="254"/>
-      <c r="F50" s="248"/>
+      <c r="A50" s="243" t="s">
+        <v>518</v>
+      </c>
+      <c r="B50" s="244" t="s">
+        <v>559</v>
+      </c>
+      <c r="C50" s="245" t="s">
+        <v>560</v>
+      </c>
+      <c r="D50" s="245"/>
+      <c r="E50" s="245"/>
+      <c r="F50" s="239"/>
     </row>
     <row r="51" spans="1:6">
-      <c r="A51" s="257" t="s">
-        <v>559</v>
+      <c r="A51" s="249" t="s">
+        <v>561</v>
       </c>
       <c r="B51" s="260"/>
       <c r="C51" s="260"/>
-      <c r="D51" s="248"/>
-      <c r="E51" s="248"/>
-      <c r="F51" s="248"/>
+      <c r="D51" s="239"/>
+      <c r="E51" s="239"/>
+      <c r="F51" s="239"/>
     </row>
     <row r="52" spans="1:6">
-      <c r="A52" s="249" t="s">
-        <v>560</v>
-      </c>
-      <c r="B52" s="250" t="s">
-        <v>561</v>
-      </c>
-      <c r="C52" s="251" t="s">
+      <c r="A52" s="240" t="s">
         <v>562</v>
       </c>
-      <c r="D52" s="251"/>
-      <c r="E52" s="251"/>
-      <c r="F52" s="248"/>
+      <c r="B52" s="241" t="s">
+        <v>563</v>
+      </c>
+      <c r="C52" s="242" t="s">
+        <v>564</v>
+      </c>
+      <c r="D52" s="242"/>
+      <c r="E52" s="242"/>
+      <c r="F52" s="239"/>
     </row>
     <row r="53" spans="1:6">
-      <c r="A53" s="252" t="s">
-        <v>563</v>
-      </c>
-      <c r="B53" s="253" t="s">
+      <c r="A53" s="243" t="s">
+        <v>565</v>
+      </c>
+      <c r="B53" s="244" t="s">
         <v>452</v>
       </c>
-      <c r="C53" s="254" t="s">
-        <v>564</v>
-      </c>
-      <c r="D53" s="254"/>
-      <c r="E53" s="254"/>
-      <c r="F53" s="248"/>
+      <c r="C53" s="245" t="s">
+        <v>566</v>
+      </c>
+      <c r="D53" s="245"/>
+      <c r="E53" s="245"/>
+      <c r="F53" s="239"/>
     </row>
     <row r="54" spans="1:6">
-      <c r="A54" s="249" t="s">
-        <v>565</v>
-      </c>
-      <c r="B54" s="250" t="s">
-        <v>566</v>
-      </c>
-      <c r="C54" s="251" t="s">
+      <c r="A54" s="240" t="s">
         <v>567</v>
       </c>
-      <c r="D54" s="251"/>
-      <c r="E54" s="251"/>
-      <c r="F54" s="248"/>
+      <c r="B54" s="241" t="s">
+        <v>568</v>
+      </c>
+      <c r="C54" s="242" t="s">
+        <v>569</v>
+      </c>
+      <c r="D54" s="242"/>
+      <c r="E54" s="242"/>
+      <c r="F54" s="239"/>
     </row>
     <row r="55" spans="1:6">
-      <c r="A55" s="252" t="s">
-        <v>568</v>
-      </c>
-      <c r="B55" s="253" t="s">
-        <v>569</v>
-      </c>
-      <c r="C55" s="254" t="s">
+      <c r="A55" s="243" t="s">
         <v>570</v>
       </c>
-      <c r="D55" s="254"/>
-      <c r="E55" s="254"/>
-      <c r="F55" s="248"/>
+      <c r="B55" s="244" t="s">
+        <v>571</v>
+      </c>
+      <c r="C55" s="245" t="s">
+        <v>572</v>
+      </c>
+      <c r="D55" s="245"/>
+      <c r="E55" s="245"/>
+      <c r="F55" s="239"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -13548,19 +13556,20 @@
     <hyperlink ref="F20" r:id="rId6" xr:uid="{83714BB7-E198-4AF2-9E3F-F0EB6C640209}"/>
     <hyperlink ref="F22" r:id="rId7" xr:uid="{3D986609-D1AD-40CD-9D91-B61C2D40A5ED}"/>
     <hyperlink ref="F23" r:id="rId8" xr:uid="{9191FE3F-DA50-42C9-A969-CB2607764014}"/>
+    <hyperlink ref="F6" r:id="rId9" xr:uid="{1A57CA13-D567-426E-8F5E-D61428112166}"/>
+    <hyperlink ref="E6" r:id="rId10" xr:uid="{AD9D2A23-197E-48AD-BEB3-D183F57E51A7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" r:id="rId9"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" r:id="rId11"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="8ee09cf5-53a8-4aeb-94af-927f54a7d6d8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -13803,15 +13812,16 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="8ee09cf5-53a8-4aeb-94af-927f54a7d6d8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8E275EF-C000-4518-B0F8-FE9A60820B51}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC6EF48D-28DC-4A85-AE0A-77598A9ABE97}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -13819,5 +13829,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC6EF48D-28DC-4A85-AE0A-77598A9ABE97}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8E275EF-C000-4518-B0F8-FE9A60820B51}"/>
 </file>
</xml_diff>

<commit_message>
Update icon config to sakura.png
</commit_message>
<xml_diff>
--- a/japantour.xlsx
+++ b/japantour.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bscvn-my.sharepoint.com/personal/minhpq_bsc_com_vn/Documents/09_CODER/00_travel-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="167" documentId="13_ncr:1_{4CBA3FCD-3F21-4F99-9320-E2DF1148D8FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD04243F-370A-43DE-9081-B5FB59FFBFE7}"/>
+  <xr:revisionPtr revIDLastSave="169" documentId="13_ncr:1_{4CBA3FCD-3F21-4F99-9320-E2DF1148D8FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB8D47EC-124B-4100-A040-E46359791ED3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="458" firstSheet="4" activeTab="4" xr2:uid="{1D34A874-FA64-408A-8A73-D0DA492D543E}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1005" uniqueCount="573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1007" uniqueCount="575">
   <si>
     <t>Đơn giá</t>
   </si>
@@ -1421,6 +1421,9 @@
     <t>Airbnb</t>
   </si>
   <si>
+    <t>1_day1_airbnb.png</t>
+  </si>
+  <si>
     <t>https://maps.app.goo.gl/DBmdvffro3LetJej6</t>
   </si>
   <si>
@@ -1461,6 +1464,9 @@
   </si>
   <si>
     <t>Miraikan</t>
+  </si>
+  <si>
+    <t>1_day1_miraikan.png</t>
   </si>
   <si>
     <t>https://maps.app.goo.gl/BmYZxEzfSyLjgQyp9</t>
@@ -12830,40 +12836,42 @@
       <c r="D5" s="242" t="s">
         <v>449</v>
       </c>
-      <c r="E5" s="242"/>
+      <c r="E5" s="8" t="s">
+        <v>450</v>
+      </c>
       <c r="F5" s="247" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="243" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B6" s="244" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C6" s="245" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D6" s="245" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="F6" s="246" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.75">
       <c r="A7" s="240" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B7" s="244" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C7" s="245" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D7" s="245"/>
       <c r="E7" s="245"/>
@@ -12871,49 +12879,51 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="243" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B8" s="244" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C8" s="245" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D8" s="245" t="s">
-        <v>463</v>
-      </c>
-      <c r="E8" s="245"/>
+        <v>464</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>465</v>
+      </c>
       <c r="F8" s="246" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="240" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B9" s="241" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="C9" s="242" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="D9" s="242" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="E9" s="242"/>
       <c r="F9" s="246" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="243" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B10" s="244" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C10" s="245" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="D10" s="245"/>
       <c r="E10" s="245"/>
@@ -12924,10 +12934,10 @@
         <v>0.875</v>
       </c>
       <c r="B11" s="241" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C11" s="242" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="D11" s="242"/>
       <c r="E11" s="242"/>
@@ -12935,7 +12945,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="249" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B12" s="260"/>
       <c r="C12" s="260"/>
@@ -12945,31 +12955,31 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="240" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B13" s="241" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="C13" s="242" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="D13" s="242" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="E13" s="242"/>
       <c r="F13" s="246" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="29.25">
       <c r="A14" s="243" t="s">
+        <v>483</v>
+      </c>
+      <c r="B14" s="244" t="s">
         <v>481</v>
       </c>
-      <c r="B14" s="244" t="s">
-        <v>479</v>
-      </c>
       <c r="C14" s="245" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="D14" s="245"/>
       <c r="E14" s="245"/>
@@ -12977,20 +12987,20 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="240" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B15" s="241" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C15" s="242" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="D15" s="242" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="E15" s="242"/>
       <c r="F15" s="246" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -12998,10 +13008,10 @@
         <v>0.875</v>
       </c>
       <c r="B16" s="241" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C16" s="242" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="D16" s="245"/>
       <c r="E16" s="245"/>
@@ -13009,7 +13019,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="249" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B17" s="260"/>
       <c r="C17" s="260"/>
@@ -13019,13 +13029,13 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="240" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B18" s="241" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="C18" s="242" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="D18" s="242"/>
       <c r="E18" s="242"/>
@@ -13033,13 +13043,13 @@
     </row>
     <row r="19" spans="1:6" ht="29.25">
       <c r="A19" s="243" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B19" s="244" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="C19" s="245" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="D19" s="245"/>
       <c r="E19" s="245"/>
@@ -13047,31 +13057,31 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="240" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B20" s="241" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C20" s="242" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="D20" s="242" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="E20" s="242"/>
       <c r="F20" s="246" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="243" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B21" s="244" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="C21" s="245" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="D21" s="245"/>
       <c r="E21" s="245"/>
@@ -13079,41 +13089,41 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="240" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B22" s="241" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="C22" s="242" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="D22" s="242" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="E22" s="242"/>
       <c r="F22" s="246" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="243" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B23" s="244" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C23" s="245" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="D23" s="245"/>
       <c r="E23" s="245"/>
       <c r="F23" s="8" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="249" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B24" s="260"/>
       <c r="C24" s="260"/>
@@ -13123,13 +13133,13 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="240" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B25" s="241" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="C25" s="242" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="D25" s="242"/>
       <c r="E25" s="242"/>
@@ -13137,13 +13147,13 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="243" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B26" s="244" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C26" s="245" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="D26" s="245"/>
       <c r="E26" s="245"/>
@@ -13151,13 +13161,13 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="240" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B27" s="241" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="C27" s="242" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="D27" s="242"/>
       <c r="E27" s="242"/>
@@ -13165,13 +13175,13 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="243" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B28" s="244" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="C28" s="245" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="D28" s="245"/>
       <c r="E28" s="245"/>
@@ -13179,13 +13189,13 @@
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="240" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B29" s="241" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="C29" s="242" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D29" s="242"/>
       <c r="E29" s="242"/>
@@ -13193,7 +13203,7 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="249" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="B30" s="260"/>
       <c r="C30" s="260"/>
@@ -13203,13 +13213,13 @@
     </row>
     <row r="31" spans="1:6" ht="29.25">
       <c r="A31" s="240" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B31" s="241" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="C31" s="242" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="D31" s="242"/>
       <c r="E31" s="242"/>
@@ -13217,13 +13227,13 @@
     </row>
     <row r="32" spans="1:6" ht="29.25">
       <c r="A32" s="243" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B32" s="244" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C32" s="245" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="D32" s="245"/>
       <c r="E32" s="245"/>
@@ -13231,13 +13241,13 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="240" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="B33" s="241" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="C33" s="242" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="D33" s="242"/>
       <c r="E33" s="242"/>
@@ -13245,13 +13255,13 @@
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="243" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B34" s="244" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C34" s="245" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D34" s="245"/>
       <c r="E34" s="245"/>
@@ -13259,7 +13269,7 @@
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="249" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="B35" s="260"/>
       <c r="C35" s="260"/>
@@ -13269,13 +13279,13 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="240" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B36" s="241" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="C36" s="242" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="D36" s="242"/>
       <c r="E36" s="242"/>
@@ -13283,13 +13293,13 @@
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="243" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B37" s="244" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C37" s="245" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="D37" s="245"/>
       <c r="E37" s="245"/>
@@ -13297,13 +13307,13 @@
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="240" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B38" s="241" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="C38" s="242" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="D38" s="242"/>
       <c r="E38" s="242"/>
@@ -13311,13 +13321,13 @@
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="243" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="B39" s="244" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="C39" s="245" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="D39" s="245"/>
       <c r="E39" s="245"/>
@@ -13325,13 +13335,13 @@
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="240" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="B40" s="241" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C40" s="242" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="D40" s="242"/>
       <c r="E40" s="242"/>
@@ -13339,7 +13349,7 @@
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="249" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="B41" s="260"/>
       <c r="C41" s="260"/>
@@ -13349,13 +13359,13 @@
     </row>
     <row r="42" spans="1:6" ht="29.25">
       <c r="A42" s="240" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B42" s="241" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="C42" s="242" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="D42" s="242"/>
       <c r="E42" s="242"/>
@@ -13363,13 +13373,13 @@
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="243" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B43" s="244" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C43" s="245" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="D43" s="245"/>
       <c r="E43" s="245"/>
@@ -13377,13 +13387,13 @@
     </row>
     <row r="44" spans="1:6">
       <c r="A44" s="240" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B44" s="241" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="C44" s="242" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="D44" s="242"/>
       <c r="E44" s="242"/>
@@ -13391,13 +13401,13 @@
     </row>
     <row r="45" spans="1:6" ht="15.75">
       <c r="A45" s="243" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="B45" s="244" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="C45" s="245" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D45" s="245"/>
       <c r="E45" s="245"/>
@@ -13405,7 +13415,7 @@
     </row>
     <row r="46" spans="1:6">
       <c r="A46" s="249" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="B46" s="260"/>
       <c r="C46" s="260"/>
@@ -13415,13 +13425,13 @@
     </row>
     <row r="47" spans="1:6" ht="29.25">
       <c r="A47" s="240" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B47" s="241" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="C47" s="242" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="D47" s="242"/>
       <c r="E47" s="242"/>
@@ -13429,13 +13439,13 @@
     </row>
     <row r="48" spans="1:6">
       <c r="A48" s="243" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B48" s="244" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C48" s="245" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="D48" s="245"/>
       <c r="E48" s="245"/>
@@ -13443,13 +13453,13 @@
     </row>
     <row r="49" spans="1:6">
       <c r="A49" s="240" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="B49" s="241" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="C49" s="242" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="D49" s="242"/>
       <c r="E49" s="242"/>
@@ -13457,13 +13467,13 @@
     </row>
     <row r="50" spans="1:6">
       <c r="A50" s="243" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B50" s="244" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="C50" s="245" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="D50" s="245"/>
       <c r="E50" s="245"/>
@@ -13471,7 +13481,7 @@
     </row>
     <row r="51" spans="1:6">
       <c r="A51" s="249" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="B51" s="260"/>
       <c r="C51" s="260"/>
@@ -13481,13 +13491,13 @@
     </row>
     <row r="52" spans="1:6">
       <c r="A52" s="240" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="B52" s="241" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="C52" s="242" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="D52" s="242"/>
       <c r="E52" s="242"/>
@@ -13495,13 +13505,13 @@
     </row>
     <row r="53" spans="1:6">
       <c r="A53" s="243" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="B53" s="244" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C53" s="245" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="D53" s="245"/>
       <c r="E53" s="245"/>
@@ -13509,13 +13519,13 @@
     </row>
     <row r="54" spans="1:6">
       <c r="A54" s="240" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="B54" s="241" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="C54" s="242" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D54" s="242"/>
       <c r="E54" s="242"/>
@@ -13523,13 +13533,13 @@
     </row>
     <row r="55" spans="1:6">
       <c r="A55" s="243" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="B55" s="244" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="C55" s="245" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="D55" s="245"/>
       <c r="E55" s="245"/>
@@ -13558,9 +13568,11 @@
     <hyperlink ref="F23" r:id="rId8" xr:uid="{9191FE3F-DA50-42C9-A969-CB2607764014}"/>
     <hyperlink ref="F6" r:id="rId9" xr:uid="{1A57CA13-D567-426E-8F5E-D61428112166}"/>
     <hyperlink ref="E6" r:id="rId10" xr:uid="{AD9D2A23-197E-48AD-BEB3-D183F57E51A7}"/>
+    <hyperlink ref="E8" r:id="rId11" xr:uid="{C57DE3BC-5611-4857-AF68-85AE0077E820}"/>
+    <hyperlink ref="E5" r:id="rId12" xr:uid="{51324F1C-9EC8-4171-933D-4D6E14F3B038}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" r:id="rId11"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" r:id="rId13"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Update polished tour itinerary
</commit_message>
<xml_diff>
--- a/japantour.xlsx
+++ b/japantour.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bscvn-my.sharepoint.com/personal/minhpq_bsc_com_vn/Documents/09_CODER/00_travel-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="247" documentId="13_ncr:1_{4CBA3FCD-3F21-4F99-9320-E2DF1148D8FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7289F77C-0872-4599-A591-E6EFF1EB460D}"/>
+  <xr:revisionPtr revIDLastSave="275" documentId="13_ncr:1_{4CBA3FCD-3F21-4F99-9320-E2DF1148D8FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{684A8C4B-AF99-47DE-9279-F7149DF921CA}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="458" activeTab="4" xr2:uid="{1D34A874-FA64-408A-8A73-D0DA492D543E}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1050" uniqueCount="617">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="629">
   <si>
     <t>Đơn giá</t>
   </si>
@@ -1700,18 +1700,12 @@
     <t>Arashiyama Sights</t>
   </si>
   <si>
-    <t>Morning stroll in Bamboo Grove, Hozu River scenic boat tour &amp; visit moss temple Otagi Nenbutsu-ji.</t>
-  </si>
-  <si>
     <t>Kyoto style Udon noodles &amp; sweets at Ogura Cha-Ya.</t>
   </si>
   <si>
     <t>Sagano Romantic Train</t>
   </si>
   <si>
-    <t>Vintage scenic train ride along Sagano romantic river gorge.</t>
-  </si>
-  <si>
     <t>17:00 - 19:30</t>
   </si>
   <si>
@@ -1920,6 +1914,48 @@
   </si>
   <si>
     <t>Kyoto farewell dinner &amp; traditional Matcha souvenir shopping. Dinner at Sukiya</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/1e471XSYSH6i2k5x8</t>
+  </si>
+  <si>
+    <t>Boat Rental Boarding</t>
+  </si>
+  <si>
+    <t>Morning stroll in Bamboo Grove &amp; visit moss temple Otagi Nenbutsu-ji.</t>
+  </si>
+  <si>
+    <t>Hozu River scenic boat tour</t>
+  </si>
+  <si>
+    <t>Bamboo Grove</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/roLsEvwaGtW57c5x5</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/dFzWPyLP4fn9B2ZR6</t>
+  </si>
+  <si>
+    <t>Pizza Restaurant</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/3M4ACDEmUwSknxXW6</t>
+  </si>
+  <si>
+    <t>Unagi Restaurant</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/jNcHH5W7jbrYFafF6</t>
+  </si>
+  <si>
+    <t>Nara Park</t>
+  </si>
+  <si>
+    <t>Gion Starbucks</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/Lcn3t16zCf3ddAAF6</t>
   </si>
 </sst>
 </file>
@@ -13070,7 +13106,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="249" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="B11" s="241" t="s">
         <v>477</v>
@@ -13100,13 +13136,13 @@
         <v>481</v>
       </c>
       <c r="C13" s="242" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="D13" s="242" t="s">
         <v>482</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="F13" s="246" t="s">
         <v>483</v>
@@ -13140,7 +13176,7 @@
         <v>488</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="F15" s="246" t="s">
         <v>489</v>
@@ -13196,7 +13232,7 @@
       </c>
       <c r="D19" s="245"/>
       <c r="E19" s="8" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="F19" s="239"/>
     </row>
@@ -13211,10 +13247,10 @@
         <v>498</v>
       </c>
       <c r="D20" s="242" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="F20" s="246" t="s">
         <v>499</v>
@@ -13248,7 +13284,7 @@
         <v>506</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="F22" s="246" t="s">
         <v>507</v>
@@ -13265,7 +13301,7 @@
         <v>508</v>
       </c>
       <c r="D23" s="245" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="E23" s="251"/>
       <c r="F23" s="8" t="s">
@@ -13290,16 +13326,16 @@
         <v>512</v>
       </c>
       <c r="C25" s="242" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="D25" s="242" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="F25" s="239" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -13310,16 +13346,16 @@
         <v>453</v>
       </c>
       <c r="C26" s="245" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="D26" s="245" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="F26" s="239" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -13333,11 +13369,11 @@
         <v>516</v>
       </c>
       <c r="D27" s="242" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="E27" s="250"/>
       <c r="F27" s="239" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -13348,16 +13384,16 @@
         <v>504</v>
       </c>
       <c r="C28" s="245" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="D28" s="245" t="s">
+        <v>577</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>596</v>
+      </c>
+      <c r="F28" s="239" t="s">
         <v>579</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>598</v>
-      </c>
-      <c r="F28" s="239" t="s">
-        <v>581</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -13371,13 +13407,13 @@
         <v>519</v>
       </c>
       <c r="D29" s="242" t="s">
+        <v>578</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>595</v>
+      </c>
+      <c r="F29" s="239" t="s">
         <v>580</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>597</v>
-      </c>
-      <c r="F29" s="239" t="s">
-        <v>582</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -13398,16 +13434,16 @@
         <v>522</v>
       </c>
       <c r="C31" s="242" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="D31" s="242" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="F31" s="239" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -13422,7 +13458,7 @@
       </c>
       <c r="D32" s="245"/>
       <c r="E32" s="8" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="F32" s="239"/>
     </row>
@@ -13451,11 +13487,11 @@
         <v>529</v>
       </c>
       <c r="D34" s="245" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="E34" s="251"/>
       <c r="F34" s="239" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -13480,7 +13516,7 @@
       </c>
       <c r="D36" s="242"/>
       <c r="E36" s="8" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="F36" s="239"/>
     </row>
@@ -13495,13 +13531,13 @@
         <v>534</v>
       </c>
       <c r="D37" s="245" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="F37" s="239" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -13516,7 +13552,7 @@
       </c>
       <c r="D38" s="242"/>
       <c r="E38" s="8" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="F38" s="239"/>
     </row>
@@ -13531,13 +13567,13 @@
         <v>538</v>
       </c>
       <c r="D39" s="242" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="F39" s="239" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -13564,7 +13600,7 @@
       <c r="E41" s="239"/>
       <c r="F41" s="239"/>
     </row>
-    <row r="42" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="240" t="s">
         <v>494</v>
       </c>
@@ -13572,13 +13608,17 @@
         <v>542</v>
       </c>
       <c r="C42" s="242" t="s">
-        <v>543</v>
-      </c>
-      <c r="D42" s="242"/>
+        <v>617</v>
+      </c>
+      <c r="D42" s="242" t="s">
+        <v>619</v>
+      </c>
       <c r="E42" s="8" t="s">
-        <v>610</v>
-      </c>
-      <c r="F42" s="239"/>
+        <v>608</v>
+      </c>
+      <c r="F42" s="239" t="s">
+        <v>620</v>
+      </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="243" t="s">
@@ -13588,7 +13628,7 @@
         <v>453</v>
       </c>
       <c r="C43" s="245" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="D43" s="245"/>
       <c r="E43" s="251"/>
@@ -13599,36 +13639,44 @@
         <v>514</v>
       </c>
       <c r="B44" s="241" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="C44" s="242" t="s">
-        <v>546</v>
-      </c>
-      <c r="D44" s="242"/>
+        <v>618</v>
+      </c>
+      <c r="D44" s="242" t="s">
+        <v>616</v>
+      </c>
       <c r="E44" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F44" s="239"/>
+        <v>609</v>
+      </c>
+      <c r="F44" s="239" t="s">
+        <v>615</v>
+      </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="243" t="s">
+        <v>545</v>
+      </c>
+      <c r="B45" s="244" t="s">
+        <v>546</v>
+      </c>
+      <c r="C45" s="245" t="s">
         <v>547</v>
       </c>
-      <c r="B45" s="244" t="s">
-        <v>548</v>
-      </c>
-      <c r="C45" s="245" t="s">
-        <v>549</v>
-      </c>
-      <c r="D45" s="245"/>
+      <c r="D45" s="245" t="s">
+        <v>622</v>
+      </c>
       <c r="E45" s="8" t="s">
-        <v>612</v>
-      </c>
-      <c r="F45" s="239"/>
+        <v>610</v>
+      </c>
+      <c r="F45" s="239" t="s">
+        <v>621</v>
+      </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="253" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="B46" s="254"/>
       <c r="C46" s="254"/>
@@ -13641,16 +13689,20 @@
         <v>531</v>
       </c>
       <c r="B47" s="241" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="C47" s="242" t="s">
-        <v>552</v>
-      </c>
-      <c r="D47" s="242"/>
+        <v>550</v>
+      </c>
+      <c r="D47" s="242" t="s">
+        <v>627</v>
+      </c>
       <c r="E47" s="8" t="s">
-        <v>613</v>
-      </c>
-      <c r="F47" s="239"/>
+        <v>611</v>
+      </c>
+      <c r="F47" s="239" t="s">
+        <v>628</v>
+      </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="243" t="s">
@@ -13660,39 +13712,47 @@
         <v>453</v>
       </c>
       <c r="C48" s="245" t="s">
-        <v>553</v>
-      </c>
-      <c r="D48" s="245"/>
+        <v>551</v>
+      </c>
+      <c r="D48" s="245" t="s">
+        <v>624</v>
+      </c>
       <c r="E48" s="8" t="s">
-        <v>614</v>
-      </c>
-      <c r="F48" s="239"/>
+        <v>612</v>
+      </c>
+      <c r="F48" s="239" t="s">
+        <v>623</v>
+      </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="240" t="s">
+        <v>552</v>
+      </c>
+      <c r="B49" s="241" t="s">
+        <v>553</v>
+      </c>
+      <c r="C49" s="242" t="s">
         <v>554</v>
       </c>
-      <c r="B49" s="241" t="s">
-        <v>555</v>
-      </c>
-      <c r="C49" s="242" t="s">
-        <v>556</v>
-      </c>
-      <c r="D49" s="242"/>
+      <c r="D49" s="242" t="s">
+        <v>626</v>
+      </c>
       <c r="E49" s="8" t="s">
-        <v>615</v>
-      </c>
-      <c r="F49" s="239"/>
+        <v>613</v>
+      </c>
+      <c r="F49" s="239" t="s">
+        <v>625</v>
+      </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="243" t="s">
         <v>517</v>
       </c>
       <c r="B50" s="244" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="C50" s="245" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="D50" s="245"/>
       <c r="E50" s="251"/>
@@ -13700,7 +13760,7 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="253" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="B51" s="254"/>
       <c r="C51" s="254"/>
@@ -13710,13 +13770,13 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="240" t="s">
+        <v>557</v>
+      </c>
+      <c r="B52" s="241" t="s">
+        <v>558</v>
+      </c>
+      <c r="C52" s="242" t="s">
         <v>559</v>
-      </c>
-      <c r="B52" s="241" t="s">
-        <v>560</v>
-      </c>
-      <c r="C52" s="242" t="s">
-        <v>561</v>
       </c>
       <c r="D52" s="242"/>
       <c r="E52" s="250"/>
@@ -13724,13 +13784,13 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="243" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="B53" s="244" t="s">
         <v>453</v>
       </c>
       <c r="C53" s="245" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="D53" s="245"/>
       <c r="E53" s="251"/>
@@ -13738,13 +13798,13 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="240" t="s">
+        <v>562</v>
+      </c>
+      <c r="B54" s="241" t="s">
+        <v>563</v>
+      </c>
+      <c r="C54" s="242" t="s">
         <v>564</v>
-      </c>
-      <c r="B54" s="241" t="s">
-        <v>565</v>
-      </c>
-      <c r="C54" s="242" t="s">
-        <v>566</v>
       </c>
       <c r="D54" s="242"/>
       <c r="E54" s="250"/>
@@ -13752,13 +13812,13 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="243" t="s">
+        <v>565</v>
+      </c>
+      <c r="B55" s="244" t="s">
+        <v>566</v>
+      </c>
+      <c r="C55" s="245" t="s">
         <v>567</v>
-      </c>
-      <c r="B55" s="244" t="s">
-        <v>568</v>
-      </c>
-      <c r="C55" s="245" t="s">
-        <v>569</v>
       </c>
       <c r="D55" s="245"/>
       <c r="E55" s="251"/>
@@ -13807,11 +13867,11 @@
     <hyperlink ref="E36" r:id="rId28" display="../../../../../:i:/g/personal/minhpq_bsc_com_vn/IQAi5aJIKv75Q5U5vm6kHBDjARkqNOrYQa7d-mPqOmt_l9M?e=odHoQX" xr:uid="{2B6E1CBF-87A2-4134-BE94-277B3CC7FFB9}"/>
     <hyperlink ref="E42" r:id="rId29" display="../../../../../:i:/g/personal/minhpq_bsc_com_vn/IQBvxNjcSnLqT7jKgOPhtaV8AWmmNNqk6oh9a1lt8vbQuno?e=btuKan" xr:uid="{38E5D752-73C6-4466-B72D-45897A20A545}"/>
     <hyperlink ref="E39" r:id="rId30" display="../../../../../:i:/g/personal/minhpq_bsc_com_vn/IQAB-UbxLXE3QalHQcXGuVhMAY7ZhR4RXior7Gu8u3jicQ4?e=iFyZcH" xr:uid="{072046B0-F592-4B21-9C7B-E122D9FE42AE}"/>
-    <hyperlink ref="E44" r:id="rId31" display="../../../../../:i:/g/personal/minhpq_bsc_com_vn/IQCMDsm-cXytSrMd_2AsKK9rAexWEsufMEj4eRK-hf43jbY?e=ki8ssH" xr:uid="{414A8FBD-C238-4CD6-8144-C94627BB946F}"/>
-    <hyperlink ref="E45" r:id="rId32" display="../../../../../:i:/g/personal/minhpq_bsc_com_vn/IQBuagFda6KEQLdJQxAPyzQIAXHRwhrheicUfs557gRiOdY?e=LeZ2a1" xr:uid="{C4EF7A10-6175-4B2C-AC44-311F983866BF}"/>
-    <hyperlink ref="E47" r:id="rId33" display="../../../../../:i:/g/personal/minhpq_bsc_com_vn/IQBFE0qgiEGLT4MoTK3gdmuTASMCfsn-oI0Q48ttZEdKGy8?e=bIP6eJ" xr:uid="{776B393A-91D9-4A8D-B892-566419B6B1BF}"/>
-    <hyperlink ref="E48" r:id="rId34" display="../../../../../:i:/g/personal/minhpq_bsc_com_vn/IQBbK0oEKOLiS6e6S3WODu0YAcall48pO6VlsUn_tzRXYBo?e=kR4APw" xr:uid="{F0B9731E-50CC-41FC-BF46-0A9929D1F4FC}"/>
-    <hyperlink ref="E49" r:id="rId35" display="../../../../../:i:/g/personal/minhpq_bsc_com_vn/IQDN3mn-pXumRq_7HUsZQPoOAT__vEn4Yk9Nx376hc7c1J0?e=uP0ehC" xr:uid="{DC3492E8-1EB1-4B3F-A764-2F78CEA84404}"/>
+    <hyperlink ref="E45" r:id="rId31" display="../../../../../:i:/g/personal/minhpq_bsc_com_vn/IQBuagFda6KEQLdJQxAPyzQIAXHRwhrheicUfs557gRiOdY?e=LeZ2a1" xr:uid="{C4EF7A10-6175-4B2C-AC44-311F983866BF}"/>
+    <hyperlink ref="E47" r:id="rId32" display="../../../../../:i:/g/personal/minhpq_bsc_com_vn/IQBFE0qgiEGLT4MoTK3gdmuTASMCfsn-oI0Q48ttZEdKGy8?e=bIP6eJ" xr:uid="{776B393A-91D9-4A8D-B892-566419B6B1BF}"/>
+    <hyperlink ref="E48" r:id="rId33" display="../../../../../:i:/g/personal/minhpq_bsc_com_vn/IQBbK0oEKOLiS6e6S3WODu0YAcall48pO6VlsUn_tzRXYBo?e=kR4APw" xr:uid="{F0B9731E-50CC-41FC-BF46-0A9929D1F4FC}"/>
+    <hyperlink ref="E49" r:id="rId34" display="../../../../../:i:/g/personal/minhpq_bsc_com_vn/IQDN3mn-pXumRq_7HUsZQPoOAT__vEn4Yk9Nx376hc7c1J0?e=uP0ehC" xr:uid="{DC3492E8-1EB1-4B3F-A764-2F78CEA84404}"/>
+    <hyperlink ref="E44" r:id="rId35" display="../../../../../:i:/g/personal/minhpq_bsc_com_vn/IQCMDsm-cXytSrMd_2AsKK9rAexWEsufMEj4eRK-hf43jbY?e=p9lxX0" xr:uid="{19EF1E07-911D-4B4A-8D8A-88DF318FF2A8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" r:id="rId36"/>

</xml_diff>

<commit_message>
Update liquid glass layout and sync all assets
</commit_message>
<xml_diff>
--- a/japantour.xlsx
+++ b/japantour.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bscvn-my.sharepoint.com/personal/minhpq_bsc_com_vn/Documents/09_CODER/00_travel-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="275" documentId="13_ncr:1_{4CBA3FCD-3F21-4F99-9320-E2DF1148D8FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{684A8C4B-AF99-47DE-9279-F7149DF921CA}"/>
+  <xr:revisionPtr revIDLastSave="276" documentId="13_ncr:1_{4CBA3FCD-3F21-4F99-9320-E2DF1148D8FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A40AFE6C-7F4F-4E73-9796-AB7F711D87F3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="458" activeTab="4" xr2:uid="{1D34A874-FA64-408A-8A73-D0DA492D543E}"/>
   </bookViews>
@@ -1703,9 +1703,6 @@
     <t>Kyoto style Udon noodles &amp; sweets at Ogura Cha-Ya.</t>
   </si>
   <si>
-    <t>Sagano Romantic Train</t>
-  </si>
-  <si>
     <t>17:00 - 19:30</t>
   </si>
   <si>
@@ -1956,6 +1953,9 @@
   </si>
   <si>
     <t>https://maps.app.goo.gl/Lcn3t16zCf3ddAAF6</t>
+  </si>
+  <si>
+    <t>Scenic Boat</t>
   </si>
 </sst>
 </file>
@@ -13106,7 +13106,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="249" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B11" s="241" t="s">
         <v>477</v>
@@ -13136,13 +13136,13 @@
         <v>481</v>
       </c>
       <c r="C13" s="242" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="D13" s="242" t="s">
         <v>482</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="F13" s="246" t="s">
         <v>483</v>
@@ -13176,7 +13176,7 @@
         <v>488</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="F15" s="246" t="s">
         <v>489</v>
@@ -13232,7 +13232,7 @@
       </c>
       <c r="D19" s="245"/>
       <c r="E19" s="8" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="F19" s="239"/>
     </row>
@@ -13247,10 +13247,10 @@
         <v>498</v>
       </c>
       <c r="D20" s="242" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F20" s="246" t="s">
         <v>499</v>
@@ -13284,7 +13284,7 @@
         <v>506</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="F22" s="246" t="s">
         <v>507</v>
@@ -13301,7 +13301,7 @@
         <v>508</v>
       </c>
       <c r="D23" s="245" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="E23" s="251"/>
       <c r="F23" s="8" t="s">
@@ -13326,16 +13326,16 @@
         <v>512</v>
       </c>
       <c r="C25" s="242" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="D25" s="242" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="F25" s="239" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -13346,16 +13346,16 @@
         <v>453</v>
       </c>
       <c r="C26" s="245" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="D26" s="245" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="F26" s="239" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -13369,11 +13369,11 @@
         <v>516</v>
       </c>
       <c r="D27" s="242" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="E27" s="250"/>
       <c r="F27" s="239" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -13384,16 +13384,16 @@
         <v>504</v>
       </c>
       <c r="C28" s="245" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="D28" s="245" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="F28" s="239" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -13407,13 +13407,13 @@
         <v>519</v>
       </c>
       <c r="D29" s="242" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="F29" s="239" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -13434,16 +13434,16 @@
         <v>522</v>
       </c>
       <c r="C31" s="242" t="s">
+        <v>583</v>
+      </c>
+      <c r="D31" s="242" t="s">
+        <v>570</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>597</v>
+      </c>
+      <c r="F31" s="239" t="s">
         <v>584</v>
-      </c>
-      <c r="D31" s="242" t="s">
-        <v>571</v>
-      </c>
-      <c r="E31" s="8" t="s">
-        <v>598</v>
-      </c>
-      <c r="F31" s="239" t="s">
-        <v>585</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -13458,7 +13458,7 @@
       </c>
       <c r="D32" s="245"/>
       <c r="E32" s="8" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="F32" s="239"/>
     </row>
@@ -13487,11 +13487,11 @@
         <v>529</v>
       </c>
       <c r="D34" s="245" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="E34" s="251"/>
       <c r="F34" s="239" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -13516,7 +13516,7 @@
       </c>
       <c r="D36" s="242"/>
       <c r="E36" s="8" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="F36" s="239"/>
     </row>
@@ -13531,13 +13531,13 @@
         <v>534</v>
       </c>
       <c r="D37" s="245" t="s">
+        <v>587</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>603</v>
+      </c>
+      <c r="F37" s="239" t="s">
         <v>588</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>604</v>
-      </c>
-      <c r="F37" s="239" t="s">
-        <v>589</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -13552,7 +13552,7 @@
       </c>
       <c r="D38" s="242"/>
       <c r="E38" s="8" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="F38" s="239"/>
     </row>
@@ -13567,13 +13567,13 @@
         <v>538</v>
       </c>
       <c r="D39" s="242" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="F39" s="239" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -13608,16 +13608,16 @@
         <v>542</v>
       </c>
       <c r="C42" s="242" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D42" s="242" t="s">
+        <v>618</v>
+      </c>
+      <c r="E42" s="8" t="s">
+        <v>607</v>
+      </c>
+      <c r="F42" s="239" t="s">
         <v>619</v>
-      </c>
-      <c r="E42" s="8" t="s">
-        <v>608</v>
-      </c>
-      <c r="F42" s="239" t="s">
-        <v>620</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -13639,44 +13639,44 @@
         <v>514</v>
       </c>
       <c r="B44" s="241" t="s">
-        <v>544</v>
+        <v>628</v>
       </c>
       <c r="C44" s="242" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D44" s="242" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="F44" s="239" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="243" t="s">
+        <v>544</v>
+      </c>
+      <c r="B45" s="244" t="s">
         <v>545</v>
       </c>
-      <c r="B45" s="244" t="s">
+      <c r="C45" s="245" t="s">
         <v>546</v>
       </c>
-      <c r="C45" s="245" t="s">
-        <v>547</v>
-      </c>
       <c r="D45" s="245" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="F45" s="239" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="253" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B46" s="254"/>
       <c r="C46" s="254"/>
@@ -13689,19 +13689,19 @@
         <v>531</v>
       </c>
       <c r="B47" s="241" t="s">
+        <v>548</v>
+      </c>
+      <c r="C47" s="242" t="s">
         <v>549</v>
       </c>
-      <c r="C47" s="242" t="s">
-        <v>550</v>
-      </c>
       <c r="D47" s="242" t="s">
+        <v>626</v>
+      </c>
+      <c r="E47" s="8" t="s">
+        <v>610</v>
+      </c>
+      <c r="F47" s="239" t="s">
         <v>627</v>
-      </c>
-      <c r="E47" s="8" t="s">
-        <v>611</v>
-      </c>
-      <c r="F47" s="239" t="s">
-        <v>628</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -13712,36 +13712,36 @@
         <v>453</v>
       </c>
       <c r="C48" s="245" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D48" s="245" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="F48" s="239" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="240" t="s">
+        <v>551</v>
+      </c>
+      <c r="B49" s="241" t="s">
         <v>552</v>
       </c>
-      <c r="B49" s="241" t="s">
+      <c r="C49" s="242" t="s">
         <v>553</v>
       </c>
-      <c r="C49" s="242" t="s">
-        <v>554</v>
-      </c>
       <c r="D49" s="242" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F49" s="239" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -13749,10 +13749,10 @@
         <v>517</v>
       </c>
       <c r="B50" s="244" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="C50" s="245" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="D50" s="245"/>
       <c r="E50" s="251"/>
@@ -13760,7 +13760,7 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="253" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B51" s="254"/>
       <c r="C51" s="254"/>
@@ -13770,13 +13770,13 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="240" t="s">
+        <v>556</v>
+      </c>
+      <c r="B52" s="241" t="s">
         <v>557</v>
       </c>
-      <c r="B52" s="241" t="s">
+      <c r="C52" s="242" t="s">
         <v>558</v>
-      </c>
-      <c r="C52" s="242" t="s">
-        <v>559</v>
       </c>
       <c r="D52" s="242"/>
       <c r="E52" s="250"/>
@@ -13784,13 +13784,13 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="243" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B53" s="244" t="s">
         <v>453</v>
       </c>
       <c r="C53" s="245" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="D53" s="245"/>
       <c r="E53" s="251"/>
@@ -13798,13 +13798,13 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="240" t="s">
+        <v>561</v>
+      </c>
+      <c r="B54" s="241" t="s">
         <v>562</v>
       </c>
-      <c r="B54" s="241" t="s">
+      <c r="C54" s="242" t="s">
         <v>563</v>
-      </c>
-      <c r="C54" s="242" t="s">
-        <v>564</v>
       </c>
       <c r="D54" s="242"/>
       <c r="E54" s="250"/>
@@ -13812,13 +13812,13 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="243" t="s">
+        <v>564</v>
+      </c>
+      <c r="B55" s="244" t="s">
         <v>565</v>
       </c>
-      <c r="B55" s="244" t="s">
+      <c r="C55" s="245" t="s">
         <v>566</v>
-      </c>
-      <c r="C55" s="245" t="s">
-        <v>567</v>
       </c>
       <c r="D55" s="245"/>
       <c r="E55" s="251"/>

</xml_diff>

<commit_message>
Optimize page load speed and liquid glass styles
</commit_message>
<xml_diff>
--- a/japantour.xlsx
+++ b/japantour.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bscvn-my.sharepoint.com/personal/minhpq_bsc_com_vn/Documents/09_CODER/00_travel-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="276" documentId="13_ncr:1_{4CBA3FCD-3F21-4F99-9320-E2DF1148D8FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A40AFE6C-7F4F-4E73-9796-AB7F711D87F3}"/>
+  <xr:revisionPtr revIDLastSave="277" documentId="13_ncr:1_{4CBA3FCD-3F21-4F99-9320-E2DF1148D8FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BF8FB36-C5D6-4C67-8474-79DCC0851529}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="458" activeTab="4" xr2:uid="{1D34A874-FA64-408A-8A73-D0DA492D543E}"/>
   </bookViews>
@@ -1394,9 +1394,6 @@
     <t>On Flight</t>
   </si>
   <si>
-    <t>Depart HAN on flight VJ 932 to NRT</t>
-  </si>
-  <si>
     <t>08:00 - 11:00</t>
   </si>
   <si>
@@ -1956,6 +1953,9 @@
   </si>
   <si>
     <t>Scenic Boat</t>
+  </si>
+  <si>
+    <t>Depart HAN on flight VJ 932 to NRT (From HAN to NRT)</t>
   </si>
 </sst>
 </file>
@@ -12970,7 +12970,7 @@
         <v>440</v>
       </c>
       <c r="C3" s="242" t="s">
-        <v>441</v>
+        <v>628</v>
       </c>
       <c r="D3" s="242"/>
       <c r="E3" s="250"/>
@@ -12978,71 +12978,71 @@
     </row>
     <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="243" t="s">
+        <v>441</v>
+      </c>
+      <c r="B4" s="244" t="s">
         <v>442</v>
       </c>
-      <c r="B4" s="244" t="s">
+      <c r="C4" s="245" t="s">
+        <v>442</v>
+      </c>
+      <c r="D4" s="245" t="s">
         <v>443</v>
-      </c>
-      <c r="C4" s="245" t="s">
-        <v>443</v>
-      </c>
-      <c r="D4" s="245" t="s">
-        <v>444</v>
       </c>
       <c r="E4" s="251"/>
       <c r="F4" s="246" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="240" t="s">
+        <v>445</v>
+      </c>
+      <c r="B5" s="241" t="s">
         <v>446</v>
       </c>
-      <c r="B5" s="241" t="s">
+      <c r="C5" s="242" t="s">
         <v>447</v>
       </c>
-      <c r="C5" s="242" t="s">
+      <c r="D5" s="242" t="s">
         <v>448</v>
       </c>
-      <c r="D5" s="242" t="s">
+      <c r="E5" s="252" t="s">
         <v>449</v>
       </c>
-      <c r="E5" s="252" t="s">
+      <c r="F5" s="247" t="s">
         <v>450</v>
-      </c>
-      <c r="F5" s="247" t="s">
-        <v>451</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="243" t="s">
+        <v>451</v>
+      </c>
+      <c r="B6" s="244" t="s">
         <v>452</v>
       </c>
-      <c r="B6" s="244" t="s">
+      <c r="C6" s="245" t="s">
         <v>453</v>
       </c>
-      <c r="C6" s="245" t="s">
+      <c r="D6" s="245" t="s">
         <v>454</v>
       </c>
-      <c r="D6" s="245" t="s">
+      <c r="E6" s="252" t="s">
         <v>455</v>
       </c>
-      <c r="E6" s="252" t="s">
+      <c r="F6" s="246" t="s">
         <v>456</v>
-      </c>
-      <c r="F6" s="246" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="240" t="s">
+        <v>457</v>
+      </c>
+      <c r="B7" s="244" t="s">
         <v>458</v>
       </c>
-      <c r="B7" s="244" t="s">
+      <c r="C7" s="245" t="s">
         <v>459</v>
-      </c>
-      <c r="C7" s="245" t="s">
-        <v>460</v>
       </c>
       <c r="D7" s="245"/>
       <c r="E7" s="251"/>
@@ -13050,69 +13050,69 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="243" t="s">
+        <v>460</v>
+      </c>
+      <c r="B8" s="244" t="s">
         <v>461</v>
       </c>
-      <c r="B8" s="244" t="s">
+      <c r="C8" s="245" t="s">
         <v>462</v>
       </c>
-      <c r="C8" s="245" t="s">
+      <c r="D8" s="245" t="s">
         <v>463</v>
       </c>
-      <c r="D8" s="245" t="s">
+      <c r="E8" s="252" t="s">
         <v>464</v>
       </c>
-      <c r="E8" s="252" t="s">
+      <c r="F8" s="246" t="s">
         <v>465</v>
-      </c>
-      <c r="F8" s="246" t="s">
-        <v>466</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="240" t="s">
+        <v>466</v>
+      </c>
+      <c r="B9" s="241" t="s">
         <v>467</v>
       </c>
-      <c r="B9" s="241" t="s">
+      <c r="C9" s="242" t="s">
         <v>468</v>
       </c>
-      <c r="C9" s="242" t="s">
+      <c r="D9" s="242" t="s">
         <v>469</v>
       </c>
-      <c r="D9" s="242" t="s">
+      <c r="E9" s="252" t="s">
         <v>470</v>
       </c>
-      <c r="E9" s="252" t="s">
+      <c r="F9" s="246" t="s">
         <v>471</v>
-      </c>
-      <c r="F9" s="246" t="s">
-        <v>472</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="243" t="s">
+        <v>472</v>
+      </c>
+      <c r="B10" s="244" t="s">
         <v>473</v>
       </c>
-      <c r="B10" s="244" t="s">
+      <c r="C10" s="245" t="s">
         <v>474</v>
-      </c>
-      <c r="C10" s="245" t="s">
-        <v>475</v>
       </c>
       <c r="D10" s="245"/>
       <c r="E10" s="252" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="F10" s="239"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="249" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B11" s="241" t="s">
+        <v>476</v>
+      </c>
+      <c r="C11" s="242" t="s">
         <v>477</v>
-      </c>
-      <c r="C11" s="242" t="s">
-        <v>478</v>
       </c>
       <c r="D11" s="242"/>
       <c r="E11" s="250"/>
@@ -13120,7 +13120,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="253" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B12" s="254"/>
       <c r="C12" s="254"/>
@@ -13130,33 +13130,33 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="240" t="s">
+        <v>479</v>
+      </c>
+      <c r="B13" s="241" t="s">
         <v>480</v>
       </c>
-      <c r="B13" s="241" t="s">
+      <c r="C13" s="242" t="s">
+        <v>571</v>
+      </c>
+      <c r="D13" s="242" t="s">
         <v>481</v>
       </c>
-      <c r="C13" s="242" t="s">
-        <v>572</v>
-      </c>
-      <c r="D13" s="242" t="s">
+      <c r="E13" s="8" t="s">
+        <v>591</v>
+      </c>
+      <c r="F13" s="246" t="s">
         <v>482</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>592</v>
-      </c>
-      <c r="F13" s="246" t="s">
-        <v>483</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="243" t="s">
+        <v>483</v>
+      </c>
+      <c r="B14" s="244" t="s">
+        <v>481</v>
+      </c>
+      <c r="C14" s="245" t="s">
         <v>484</v>
-      </c>
-      <c r="B14" s="244" t="s">
-        <v>482</v>
-      </c>
-      <c r="C14" s="245" t="s">
-        <v>485</v>
       </c>
       <c r="D14" s="245"/>
       <c r="E14" s="251"/>
@@ -13164,22 +13164,22 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="240" t="s">
+        <v>485</v>
+      </c>
+      <c r="B15" s="241" t="s">
+        <v>473</v>
+      </c>
+      <c r="C15" s="242" t="s">
         <v>486</v>
       </c>
-      <c r="B15" s="241" t="s">
-        <v>474</v>
-      </c>
-      <c r="C15" s="242" t="s">
+      <c r="D15" s="242" t="s">
         <v>487</v>
       </c>
-      <c r="D15" s="242" t="s">
+      <c r="E15" s="8" t="s">
+        <v>592</v>
+      </c>
+      <c r="F15" s="246" t="s">
         <v>488</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>593</v>
-      </c>
-      <c r="F15" s="246" t="s">
-        <v>489</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -13187,10 +13187,10 @@
         <v>0.875</v>
       </c>
       <c r="B16" s="241" t="s">
+        <v>476</v>
+      </c>
+      <c r="C16" s="242" t="s">
         <v>477</v>
-      </c>
-      <c r="C16" s="242" t="s">
-        <v>478</v>
       </c>
       <c r="D16" s="245"/>
       <c r="E16" s="251"/>
@@ -13198,7 +13198,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="253" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B17" s="254"/>
       <c r="C17" s="254"/>
@@ -13208,13 +13208,13 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="240" t="s">
+        <v>490</v>
+      </c>
+      <c r="B18" s="241" t="s">
         <v>491</v>
       </c>
-      <c r="B18" s="241" t="s">
+      <c r="C18" s="242" t="s">
         <v>492</v>
-      </c>
-      <c r="C18" s="242" t="s">
-        <v>493</v>
       </c>
       <c r="D18" s="242"/>
       <c r="E18" s="250"/>
@@ -13222,49 +13222,49 @@
     </row>
     <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="243" t="s">
+        <v>493</v>
+      </c>
+      <c r="B19" s="244" t="s">
         <v>494</v>
       </c>
-      <c r="B19" s="244" t="s">
+      <c r="C19" s="245" t="s">
         <v>495</v>
-      </c>
-      <c r="C19" s="245" t="s">
-        <v>496</v>
       </c>
       <c r="D19" s="245"/>
       <c r="E19" s="8" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="F19" s="239"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="240" t="s">
+        <v>496</v>
+      </c>
+      <c r="B20" s="241" t="s">
+        <v>452</v>
+      </c>
+      <c r="C20" s="242" t="s">
         <v>497</v>
       </c>
-      <c r="B20" s="241" t="s">
-        <v>453</v>
-      </c>
-      <c r="C20" s="242" t="s">
+      <c r="D20" s="242" t="s">
+        <v>572</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>598</v>
+      </c>
+      <c r="F20" s="246" t="s">
         <v>498</v>
-      </c>
-      <c r="D20" s="242" t="s">
-        <v>573</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>599</v>
-      </c>
-      <c r="F20" s="246" t="s">
-        <v>499</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="243" t="s">
+        <v>499</v>
+      </c>
+      <c r="B21" s="244" t="s">
         <v>500</v>
       </c>
-      <c r="B21" s="244" t="s">
+      <c r="C21" s="245" t="s">
         <v>501</v>
-      </c>
-      <c r="C21" s="245" t="s">
-        <v>502</v>
       </c>
       <c r="D21" s="245"/>
       <c r="E21" s="251"/>
@@ -13272,45 +13272,45 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="240" t="s">
+        <v>502</v>
+      </c>
+      <c r="B22" s="241" t="s">
         <v>503</v>
       </c>
-      <c r="B22" s="241" t="s">
+      <c r="C22" s="242" t="s">
         <v>504</v>
       </c>
-      <c r="C22" s="242" t="s">
+      <c r="D22" s="242" t="s">
         <v>505</v>
       </c>
-      <c r="D22" s="242" t="s">
+      <c r="E22" s="8" t="s">
+        <v>597</v>
+      </c>
+      <c r="F22" s="246" t="s">
         <v>506</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>598</v>
-      </c>
-      <c r="F22" s="246" t="s">
-        <v>507</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="243" t="s">
+        <v>472</v>
+      </c>
+      <c r="B23" s="244" t="s">
         <v>473</v>
       </c>
-      <c r="B23" s="244" t="s">
-        <v>474</v>
-      </c>
       <c r="C23" s="245" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="D23" s="245" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E23" s="251"/>
       <c r="F23" s="8" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="253" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B24" s="254"/>
       <c r="C24" s="254"/>
@@ -13320,105 +13320,105 @@
     </row>
     <row r="25" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="240" t="s">
+        <v>510</v>
+      </c>
+      <c r="B25" s="241" t="s">
         <v>511</v>
       </c>
-      <c r="B25" s="241" t="s">
-        <v>512</v>
-      </c>
       <c r="C25" s="242" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="D25" s="242" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="F25" s="239" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="243" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B26" s="244" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C26" s="245" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="D26" s="245" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="F26" s="239" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="240" t="s">
+        <v>513</v>
+      </c>
+      <c r="B27" s="241" t="s">
         <v>514</v>
       </c>
-      <c r="B27" s="241" t="s">
+      <c r="C27" s="242" t="s">
         <v>515</v>
       </c>
-      <c r="C27" s="242" t="s">
-        <v>516</v>
-      </c>
       <c r="D27" s="242" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="E27" s="250"/>
       <c r="F27" s="239" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="243" t="s">
+        <v>502</v>
+      </c>
+      <c r="B28" s="244" t="s">
         <v>503</v>
       </c>
-      <c r="B28" s="244" t="s">
-        <v>504</v>
-      </c>
       <c r="C28" s="245" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="D28" s="245" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="F28" s="239" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="240" t="s">
+        <v>516</v>
+      </c>
+      <c r="B29" s="241" t="s">
         <v>517</v>
       </c>
-      <c r="B29" s="241" t="s">
+      <c r="C29" s="242" t="s">
         <v>518</v>
       </c>
-      <c r="C29" s="242" t="s">
-        <v>519</v>
-      </c>
       <c r="D29" s="242" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="F29" s="239" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="253" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B30" s="254"/>
       <c r="C30" s="254"/>
@@ -13428,49 +13428,49 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="240" t="s">
+        <v>520</v>
+      </c>
+      <c r="B31" s="241" t="s">
         <v>521</v>
       </c>
-      <c r="B31" s="241" t="s">
-        <v>522</v>
-      </c>
       <c r="C31" s="242" t="s">
+        <v>582</v>
+      </c>
+      <c r="D31" s="242" t="s">
+        <v>569</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>596</v>
+      </c>
+      <c r="F31" s="239" t="s">
         <v>583</v>
-      </c>
-      <c r="D31" s="242" t="s">
-        <v>570</v>
-      </c>
-      <c r="E31" s="8" t="s">
-        <v>597</v>
-      </c>
-      <c r="F31" s="239" t="s">
-        <v>584</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="243" t="s">
+        <v>522</v>
+      </c>
+      <c r="B32" s="244" t="s">
         <v>523</v>
       </c>
-      <c r="B32" s="244" t="s">
+      <c r="C32" s="245" t="s">
         <v>524</v>
-      </c>
-      <c r="C32" s="245" t="s">
-        <v>525</v>
       </c>
       <c r="D32" s="245"/>
       <c r="E32" s="8" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="F32" s="239"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="240" t="s">
+        <v>525</v>
+      </c>
+      <c r="B33" s="241" t="s">
         <v>526</v>
       </c>
-      <c r="B33" s="241" t="s">
+      <c r="C33" s="242" t="s">
         <v>527</v>
-      </c>
-      <c r="C33" s="242" t="s">
-        <v>528</v>
       </c>
       <c r="D33" s="242"/>
       <c r="E33" s="250"/>
@@ -13478,25 +13478,25 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="243" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B34" s="244" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C34" s="245" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="D34" s="245" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="E34" s="251"/>
       <c r="F34" s="239" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="253" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B35" s="254"/>
       <c r="C35" s="254"/>
@@ -13506,85 +13506,85 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="240" t="s">
+        <v>530</v>
+      </c>
+      <c r="B36" s="241" t="s">
         <v>531</v>
       </c>
-      <c r="B36" s="241" t="s">
+      <c r="C36" s="242" t="s">
         <v>532</v>
-      </c>
-      <c r="C36" s="242" t="s">
-        <v>533</v>
       </c>
       <c r="D36" s="242"/>
       <c r="E36" s="8" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="F36" s="239"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="243" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B37" s="244" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C37" s="245" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D37" s="245" t="s">
+        <v>586</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>602</v>
+      </c>
+      <c r="F37" s="239" t="s">
         <v>587</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>603</v>
-      </c>
-      <c r="F37" s="239" t="s">
-        <v>588</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="240" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B38" s="241" t="s">
+        <v>534</v>
+      </c>
+      <c r="C38" s="242" t="s">
         <v>535</v>
-      </c>
-      <c r="C38" s="242" t="s">
-        <v>536</v>
       </c>
       <c r="D38" s="242"/>
       <c r="E38" s="8" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="F38" s="239"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="243" t="s">
+        <v>536</v>
+      </c>
+      <c r="B39" s="244" t="s">
+        <v>503</v>
+      </c>
+      <c r="C39" s="245" t="s">
         <v>537</v>
       </c>
-      <c r="B39" s="244" t="s">
-        <v>504</v>
-      </c>
-      <c r="C39" s="245" t="s">
-        <v>538</v>
-      </c>
       <c r="D39" s="242" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="F39" s="239" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="240" t="s">
+        <v>538</v>
+      </c>
+      <c r="B40" s="241" t="s">
+        <v>473</v>
+      </c>
+      <c r="C40" s="242" t="s">
         <v>539</v>
-      </c>
-      <c r="B40" s="241" t="s">
-        <v>474</v>
-      </c>
-      <c r="C40" s="242" t="s">
-        <v>540</v>
       </c>
       <c r="D40" s="242"/>
       <c r="E40" s="8"/>
@@ -13592,7 +13592,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="253" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B41" s="254"/>
       <c r="C41" s="254"/>
@@ -13602,33 +13602,33 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="240" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B42" s="241" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="C42" s="242" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D42" s="242" t="s">
+        <v>617</v>
+      </c>
+      <c r="E42" s="8" t="s">
+        <v>606</v>
+      </c>
+      <c r="F42" s="239" t="s">
         <v>618</v>
-      </c>
-      <c r="E42" s="8" t="s">
-        <v>607</v>
-      </c>
-      <c r="F42" s="239" t="s">
-        <v>619</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="243" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B43" s="244" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C43" s="245" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="D43" s="245"/>
       <c r="E43" s="251"/>
@@ -13636,47 +13636,47 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="240" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B44" s="241" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="C44" s="242" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D44" s="242" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="F44" s="239" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="243" t="s">
+        <v>543</v>
+      </c>
+      <c r="B45" s="244" t="s">
         <v>544</v>
       </c>
-      <c r="B45" s="244" t="s">
+      <c r="C45" s="245" t="s">
         <v>545</v>
       </c>
-      <c r="C45" s="245" t="s">
-        <v>546</v>
-      </c>
       <c r="D45" s="245" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="F45" s="239" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="253" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B46" s="254"/>
       <c r="C46" s="254"/>
@@ -13686,73 +13686,73 @@
     </row>
     <row r="47" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="240" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B47" s="241" t="s">
+        <v>547</v>
+      </c>
+      <c r="C47" s="242" t="s">
         <v>548</v>
       </c>
-      <c r="C47" s="242" t="s">
-        <v>549</v>
-      </c>
       <c r="D47" s="242" t="s">
+        <v>625</v>
+      </c>
+      <c r="E47" s="8" t="s">
+        <v>609</v>
+      </c>
+      <c r="F47" s="239" t="s">
         <v>626</v>
-      </c>
-      <c r="E47" s="8" t="s">
-        <v>610</v>
-      </c>
-      <c r="F47" s="239" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="243" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B48" s="244" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C48" s="245" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="D48" s="245" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="F48" s="239" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="240" t="s">
+        <v>550</v>
+      </c>
+      <c r="B49" s="241" t="s">
         <v>551</v>
       </c>
-      <c r="B49" s="241" t="s">
+      <c r="C49" s="242" t="s">
         <v>552</v>
       </c>
-      <c r="C49" s="242" t="s">
-        <v>553</v>
-      </c>
       <c r="D49" s="242" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="F49" s="239" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="243" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B50" s="244" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="C50" s="245" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="D50" s="245"/>
       <c r="E50" s="251"/>
@@ -13760,7 +13760,7 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="253" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B51" s="254"/>
       <c r="C51" s="254"/>
@@ -13770,13 +13770,13 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="240" t="s">
+        <v>555</v>
+      </c>
+      <c r="B52" s="241" t="s">
         <v>556</v>
       </c>
-      <c r="B52" s="241" t="s">
+      <c r="C52" s="242" t="s">
         <v>557</v>
-      </c>
-      <c r="C52" s="242" t="s">
-        <v>558</v>
       </c>
       <c r="D52" s="242"/>
       <c r="E52" s="250"/>
@@ -13784,13 +13784,13 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="243" t="s">
+        <v>558</v>
+      </c>
+      <c r="B53" s="244" t="s">
+        <v>452</v>
+      </c>
+      <c r="C53" s="245" t="s">
         <v>559</v>
-      </c>
-      <c r="B53" s="244" t="s">
-        <v>453</v>
-      </c>
-      <c r="C53" s="245" t="s">
-        <v>560</v>
       </c>
       <c r="D53" s="245"/>
       <c r="E53" s="251"/>
@@ -13798,13 +13798,13 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="240" t="s">
+        <v>560</v>
+      </c>
+      <c r="B54" s="241" t="s">
         <v>561</v>
       </c>
-      <c r="B54" s="241" t="s">
+      <c r="C54" s="242" t="s">
         <v>562</v>
-      </c>
-      <c r="C54" s="242" t="s">
-        <v>563</v>
       </c>
       <c r="D54" s="242"/>
       <c r="E54" s="250"/>
@@ -13812,13 +13812,13 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="243" t="s">
+        <v>563</v>
+      </c>
+      <c r="B55" s="244" t="s">
         <v>564</v>
       </c>
-      <c r="B55" s="244" t="s">
+      <c r="C55" s="245" t="s">
         <v>565</v>
-      </c>
-      <c r="C55" s="245" t="s">
-        <v>566</v>
       </c>
       <c r="D55" s="245"/>
       <c r="E55" s="251"/>
@@ -13879,6 +13879,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="8ee09cf5-53a8-4aeb-94af-927f54a7d6d8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005A4695005C4BEE4A8751FEE2C473E10D" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="df7fcaa21f93254d26451ff7a6d04ad2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="8ee09cf5-53a8-4aeb-94af-927f54a7d6d8" xmlns:ns4="ecf1487c-a58a-4bc0-a420-fb42a2a3dfc7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fefbcb393e90fe08e3723c038b505a33" ns3:_="" ns4:_="">
     <xsd:import namespace="8ee09cf5-53a8-4aeb-94af-927f54a7d6d8"/>
@@ -14117,38 +14134,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="8ee09cf5-53a8-4aeb-94af-927f54a7d6d8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A59486CE-8728-40BE-973B-B64C7CD06C40}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8E275EF-C000-4518-B0F8-FE9A60820B51}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="8ee09cf5-53a8-4aeb-94af-927f54a7d6d8"/>
-    <ds:schemaRef ds:uri="ecf1487c-a58a-4bc0-a420-fb42a2a3dfc7"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -14171,9 +14160,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8E275EF-C000-4518-B0F8-FE9A60820B51}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A59486CE-8728-40BE-973B-B64C7CD06C40}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="8ee09cf5-53a8-4aeb-94af-927f54a7d6d8"/>
+    <ds:schemaRef ds:uri="ecf1487c-a58a-4bc0-a420-fb42a2a3dfc7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>